<commit_message>
docs(qa): record genuine test execution results, defects, and feature coverage in QA workbook
</commit_message>
<xml_diff>
--- a/Job_Portal_QA_Testing_Workbook.xlsx
+++ b/Job_Portal_QA_Testing_Workbook.xlsx
@@ -909,7 +909,7 @@
       </c>
       <c r="E4">
         <f>COUNTIF('Test Cases'!$L$5:$L$213,D4)</f>
-        <v>205</v>
+        <v>192</v>
       </c>
     </row>
     <row r="5">
@@ -918,14 +918,14 @@
       </c>
       <c r="B5">
         <f>COUNTIF('Test Cases'!$L$5:$L$213,"&lt;&gt;Not Run")-COUNTIF('Test Cases'!$L$5:$L$213,"Not Applicable")</f>
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D5" t="str">
         <v>Fail</v>
       </c>
       <c r="E5">
         <f>COUNTIF('Test Cases'!$L$5:$L$213,D5)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -934,14 +934,14 @@
       </c>
       <c r="B6">
         <f>COUNTIF('Test Cases'!$L$5:$L$213,"Pass")</f>
-        <v>205</v>
+        <v>192</v>
       </c>
       <c r="D6" t="str">
         <v>Blocked</v>
       </c>
       <c r="E6">
         <f>COUNTIF('Test Cases'!$L$5:$L$213,D6)</f>
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -950,7 +950,7 @@
       </c>
       <c r="B7">
         <f>COUNTIF('Test Cases'!$L$5:$L$213,"Fail")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D7" t="str">
         <v>Not Run</v>
@@ -966,14 +966,14 @@
       </c>
       <c r="B8">
         <f>COUNTIF('Test Cases'!$L$5:$L$213,"Blocked")</f>
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="D8" t="str">
-        <v>N/A</v>
+        <v>Not Applicable</v>
       </c>
       <c r="E8">
         <f>COUNTIF('Test Cases'!$L$5:$L$213,D8)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -991,7 +991,7 @@
       </c>
       <c r="B10">
         <f>COUNTIF('Test Cases'!$L$5:$L$213,"Not Applicable")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="B11">
         <f>IF(B5=0,0,B6/B5)</f>
-        <v>1</v>
+        <v>0.9458128078817734</v>
       </c>
       <c r="D11" t="str">
         <v>Open Defect Severity</v>
@@ -1030,14 +1030,14 @@
       </c>
       <c r="B13">
         <f>COUNTIF('Bug Log'!$A$5:$A$104,"?*")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D13" t="str">
         <v>High</v>
       </c>
       <c r="E13">
         <f>COUNTIFS('Bug Log'!$E$5:$E$104,"&lt;&gt;",'Bug Log'!$K$5:$K$104,D13,'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="B14">
         <f>COUNTIFS('Bug Log'!$A$5:$A$104,"?*",'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="str">
         <v>Medium</v>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="B15">
         <f>COUNTIFS('Bug Log'!$A$5:$A$104,"?*",'Bug Log'!$K$5:$K$104,"Critical",'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")+COUNTIFS('Bug Log'!$A$5:$A$104,"?*",'Bug Log'!$K$5:$K$104,"High",'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="str">
         <v>Low</v>
@@ -9638,19 +9638,22 @@
         <v>Account is created and confirmation is shown.</v>
       </c>
       <c r="J5" t="str">
-        <v>Verified: Create account with valid details. Account is created and confirmation is shown.</v>
+        <v>Outbound delivery failure on live production: OTP SMS/Email does not arrive in user inbox due to unconfigured Resend/Twilio production keys. Only sandbox on-screen code is provided.</v>
       </c>
       <c r="K5" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>Candidate Mobile (+919876543210) &amp; Email</v>
       </c>
       <c r="L5" t="str">
-        <v>Pass</v>
+        <v>Fail</v>
+      </c>
+      <c r="M5" t="str">
+        <v>BUG-001</v>
       </c>
       <c r="N5" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O5" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/api/auth/otp/send</v>
       </c>
       <c r="P5" t="str">
         <v>Core</v>
@@ -9685,10 +9688,10 @@
         <v>Duplicate account is prevented and a clear validation message is shown.</v>
       </c>
       <c r="J6" t="str">
-        <v>Verified: Prevent duplicate account. Duplicate account is prevented and a clear validation message is shown.</v>
+        <v>Verified: Supabase Auth blocks duplicate signup with "User already registered" message.</v>
       </c>
       <c r="K6" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>existing.user@gmail.com</v>
       </c>
       <c r="L6" t="str">
         <v>Pass</v>
@@ -9697,7 +9700,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O6" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/auth</v>
       </c>
       <c r="P6" t="str">
         <v>Core</v>
@@ -9732,10 +9735,10 @@
         <v>Invalid email is rejected with clear message.</v>
       </c>
       <c r="J7" t="str">
-        <v>Verified: Validate email format. Invalid email is rejected with clear message.</v>
+        <v>Verified: HTML5 type="email" and regex validation in handleSendOtp reject "a@" and malformed email strings before submission.</v>
       </c>
       <c r="K7" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>a@, test@invalid</v>
       </c>
       <c r="L7" t="str">
         <v>Pass</v>
@@ -9744,7 +9747,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O7" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/components/AuthModal.tsx</v>
       </c>
       <c r="P7" t="str">
         <v>Core</v>
@@ -9779,10 +9782,10 @@
         <v>Mandatory fields are highlighted and submission is blocked.</v>
       </c>
       <c r="J8" t="str">
-        <v>Verified: Reject blank mandatory fields. Mandatory fields are highlighted and submission is blocked.</v>
+        <v>Verified: Submitting blank input triggers error toast: "Please enter your 10-digit mobile number or email address."</v>
       </c>
       <c r="K8" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>Empty identifier string</v>
       </c>
       <c r="L8" t="str">
         <v>Pass</v>
@@ -9791,7 +9794,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O8" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/components/AuthModal.tsx</v>
       </c>
       <c r="P8" t="str">
         <v>Core</v>
@@ -9826,10 +9829,10 @@
         <v>Rules are enforced consistently.</v>
       </c>
       <c r="J9" t="str">
-        <v>Verified: Validate minimum/maximum password rules. Rules are enforced consistently.</v>
+        <v>Verified: Supabase Auth enforces minimum 6-character password length; shorter passwords rejected with "Password should be at least 6 characters".</v>
       </c>
       <c r="K9" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>pwd="123" (&lt;6 chars)</v>
       </c>
       <c r="L9" t="str">
         <v>Pass</v>
@@ -9838,7 +9841,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O9" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/auth</v>
       </c>
       <c r="P9" t="str">
         <v>Core</v>
@@ -9873,19 +9876,19 @@
         <v>Submission is blocked with mismatch message.</v>
       </c>
       <c r="J10" t="str">
-        <v>Verified: Prevent mismatch. Submission is blocked with mismatch message.</v>
+        <v>Not Applicable: AuthModal signup form does not include a "Confirm Password" input field (only Email and Password).</v>
       </c>
       <c r="K10" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>N/A</v>
       </c>
       <c r="L10" t="str">
-        <v>Pass</v>
+        <v>Not Applicable</v>
       </c>
       <c r="N10" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O10" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/components/AuthModal.tsx:195</v>
       </c>
       <c r="P10" t="str">
         <v>Core</v>
@@ -9920,16 +9923,13 @@
         <v>OTP is accepted and verification succeeds.</v>
       </c>
       <c r="J11" t="str">
-        <v>Verification logic validates 6-digit code correctly. Outbound delivery issue tracked separately under BUG-001.</v>
+        <v>Verified: Entering the exact 6-digit OTP code in the verification modal successfully creates candidate session and returns assigned referral code.</v>
       </c>
       <c r="K11" t="str">
-        <v>6-digit OTP code</v>
+        <v>6-digit valid code</v>
       </c>
       <c r="L11" t="str">
         <v>Pass</v>
-      </c>
-      <c r="M11" t="str">
-        <v>BUG-001</v>
       </c>
       <c r="N11" t="str">
         <v>2026-09-28</v>
@@ -9970,10 +9970,10 @@
         <v>Verification fails without logging user in.</v>
       </c>
       <c r="J12" t="str">
-        <v>Verified: Reject wrong OTP. Verification fails without logging user in.</v>
+        <v>Verified: Deliberately submitting incorrect OTP returns HTTP 400 with "Incorrect OTP code. Please try again." No session created.</v>
       </c>
       <c r="K12" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>000000, 123456</v>
       </c>
       <c r="L12" t="str">
         <v>Pass</v>
@@ -9982,7 +9982,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O12" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/api/auth/otp/verify</v>
       </c>
       <c r="P12" t="str">
         <v>Core</v>
@@ -10017,10 +10017,10 @@
         <v>Expired OTP is rejected and user can request a new OTP.</v>
       </c>
       <c r="J13" t="str">
-        <v>Verified: Reject expired OTP. Expired OTP is rejected and user can request a new OTP.</v>
+        <v>Verified: In-memory OTP store enforces 5-minute (300s) TTL; expired OTP attempts return 400 "Invalid or expired OTP code".</v>
       </c>
       <c r="K13" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>OTP &gt; 300s old</v>
       </c>
       <c r="L13" t="str">
         <v>Pass</v>
@@ -10029,7 +10029,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O13" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>lib/otpStore.ts:55</v>
       </c>
       <c r="P13" t="str">
         <v>Core</v>
@@ -10064,10 +10064,10 @@
         <v>System applies defined rate limit/cooldown.</v>
       </c>
       <c r="J14" t="str">
-        <v>Verified: Prevent OTP abuse. System applies defined rate limit/cooldown.</v>
+        <v>Verified: Resend OTP button enforces a 60-second client-side countdown timer and server-side rate limit.</v>
       </c>
       <c r="K14" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>Rapid resend clicks</v>
       </c>
       <c r="L14" t="str">
         <v>Pass</v>
@@ -10076,7 +10076,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O14" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/components/AuthModal.tsx:66</v>
       </c>
       <c r="P14" t="str">
         <v>Core</v>
@@ -10111,10 +10111,10 @@
         <v>User is authenticated and lands on the correct page.</v>
       </c>
       <c r="J15" t="str">
-        <v>Verified: Login with valid credentials. User is authenticated and lands on the correct page.</v>
+        <v>Verified: Entering registered email and password authenticates user, establishes session, and closes modal.</v>
       </c>
       <c r="K15" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>registered email + valid password</v>
       </c>
       <c r="L15" t="str">
         <v>Pass</v>
@@ -10123,7 +10123,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O15" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/auth</v>
       </c>
       <c r="P15" t="str">
         <v>Core</v>
@@ -10158,10 +10158,10 @@
         <v>Login fails with generic/correct error.</v>
       </c>
       <c r="J16" t="str">
-        <v>Verified: Reject bad password. Login fails with generic/correct error.</v>
+        <v>Verified: Wrong password returns "Invalid login credentials" from Supabase Auth without logging in.</v>
       </c>
       <c r="K16" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>valid email + wrong password</v>
       </c>
       <c r="L16" t="str">
         <v>Pass</v>
@@ -10170,7 +10170,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O16" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/auth</v>
       </c>
       <c r="P16" t="str">
         <v>Core</v>
@@ -10205,10 +10205,10 @@
         <v>Login fails safely without leaking account details.</v>
       </c>
       <c r="J17" t="str">
-        <v>Verified: Handle unknown user. Login fails safely without leaking account details.</v>
+        <v>Verified: Unregistered email returns generic "Invalid login credentials" error, preventing user enumeration.</v>
       </c>
       <c r="K17" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>nonexistent_test_account_99@gmail.com</v>
       </c>
       <c r="L17" t="str">
         <v>Pass</v>
@@ -10217,7 +10217,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O17" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/auth</v>
       </c>
       <c r="P17" t="str">
         <v>Core</v>
@@ -10252,10 +10252,10 @@
         <v>Submission blocked and fields validated.</v>
       </c>
       <c r="J18" t="str">
-        <v>Verified: Validate login fields. Submission blocked and fields validated.</v>
+        <v>Verified: Blank email or password input prevented by HTML5 `required` attribute and React state guards.</v>
       </c>
       <c r="K18" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>Blank fields</v>
       </c>
       <c r="L18" t="str">
         <v>Pass</v>
@@ -10264,7 +10264,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O18" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/components/AuthModal.tsx</v>
       </c>
       <c r="P18" t="str">
         <v>Core</v>
@@ -10299,10 +10299,10 @@
         <v>Session is ended and protected pages require login.</v>
       </c>
       <c r="J19" t="str">
-        <v>Verified: End authenticated session. Session is ended and protected pages require login.</v>
+        <v>Verified: Clicking Logout clears candidate/employer session from localStorage and cookies, resetting navbar state.</v>
       </c>
       <c r="K19" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>Logout button click</v>
       </c>
       <c r="L19" t="str">
         <v>Pass</v>
@@ -10311,7 +10311,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O19" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/lib/authSession.ts:clearCandidateSession()</v>
       </c>
       <c r="P19" t="str">
         <v>Core</v>
@@ -10346,10 +10346,10 @@
         <v>Protected content is not accessible from cached session state.</v>
       </c>
       <c r="J20" t="str">
-        <v>Verified: Prevent access through browser cache. Protected content is not accessible from cached session state.</v>
+        <v>Verified: Protected dashboards (`/dashboard`, `/employer/dashboard`) check session on mount and redirect to home if logged out.</v>
       </c>
       <c r="K20" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>Browser Back button post-logout</v>
       </c>
       <c r="L20" t="str">
         <v>Pass</v>
@@ -10358,7 +10358,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O20" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/dashboard/page.tsx:28</v>
       </c>
       <c r="P20" t="str">
         <v>Core</v>
@@ -10393,10 +10393,10 @@
         <v>User is logged out or prompted to re-authenticate.</v>
       </c>
       <c r="J21" t="str">
-        <v>Verified: Expire inactive session. User is logged out or prompted to re-authenticate.</v>
+        <v>Verified: Client auth session enforces a 2.5-hour maximum lifespan (`SESSION_EXPIRY_MS = 2.5 * 60 * 60 * 1000`) before requiring re-auth.</v>
       </c>
       <c r="K21" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>Timestamp &gt; 2.5 hrs</v>
       </c>
       <c r="L21" t="str">
         <v>Pass</v>
@@ -10405,7 +10405,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O21" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/lib/authSession.ts:10</v>
       </c>
       <c r="P21" t="str">
         <v>Core</v>
@@ -10440,10 +10440,10 @@
         <v>Behavior matches product rule; no unintended session leak.</v>
       </c>
       <c r="J22" t="str">
-        <v>Verified: Validate multiple logins. Behavior matches product rule; no unintended session leak.</v>
+        <v>Verified: Dual logins from desktop and mobile browser maintain separate valid JWT tokens in Supabase.</v>
       </c>
       <c r="K22" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>Chrome desktop + Android mobile</v>
       </c>
       <c r="L22" t="str">
         <v>Pass</v>
@@ -10452,7 +10452,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O22" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/dashboard</v>
       </c>
       <c r="P22" t="str">
         <v>Core</v>
@@ -10487,19 +10487,19 @@
         <v>Password is reset successfully.</v>
       </c>
       <c r="J23" t="str">
-        <v>Verified: Reset password. Password is reset successfully.</v>
+        <v>Blocked / Not Implemented: AuthModal does not contain a "Forgot Password" link or self-service password reset email request form.</v>
       </c>
       <c r="K23" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>N/A</v>
       </c>
       <c r="L23" t="str">
-        <v>Pass</v>
+        <v>Blocked</v>
       </c>
       <c r="N23" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O23" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/components/AuthModal.tsx</v>
       </c>
       <c r="P23" t="str">
         <v>Core</v>
@@ -10534,19 +10534,19 @@
         <v>Reset is blocked and user can request a new link.</v>
       </c>
       <c r="J24" t="str">
-        <v>Verified: Reject expired reset link. Reset is blocked and user can request a new link.</v>
+        <v>Blocked / Not Implemented: No self-service password reset token flow implemented in frontend.</v>
       </c>
       <c r="K24" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>N/A</v>
       </c>
       <c r="L24" t="str">
-        <v>Pass</v>
+        <v>Blocked</v>
       </c>
       <c r="N24" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O24" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/components/AuthModal.tsx</v>
       </c>
       <c r="P24" t="str">
         <v>Core</v>
@@ -10581,19 +10581,19 @@
         <v>Reset is blocked.</v>
       </c>
       <c r="J25" t="str">
-        <v>Verified: Reject tampered reset token. Reset is blocked.</v>
+        <v>Blocked / Not Implemented: Password reset token endpoint not exposed in current App Router routes.</v>
       </c>
       <c r="K25" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>N/A</v>
       </c>
       <c r="L25" t="str">
-        <v>Pass</v>
+        <v>Blocked</v>
       </c>
       <c r="N25" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O25" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/api/auth/*</v>
       </c>
       <c r="P25" t="str">
         <v>Core</v>
@@ -10628,19 +10628,19 @@
         <v>Change is rejected.</v>
       </c>
       <c r="J26" t="str">
-        <v>Verified: Validate current password. Change is rejected.</v>
+        <v>Blocked / Not Implemented: Candidate dashboard does not have an in-app "Change Password" form requiring current password.</v>
       </c>
       <c r="K26" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>N/A</v>
       </c>
       <c r="L26" t="str">
-        <v>Pass</v>
+        <v>Blocked</v>
       </c>
       <c r="N26" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O26" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/dashboard/page.tsx</v>
       </c>
       <c r="P26" t="str">
         <v>Core</v>
@@ -10675,19 +10675,19 @@
         <v>Password display toggles without altering value.</v>
       </c>
       <c r="J27" t="str">
-        <v>Verified: Show/hide password. Password display toggles without altering value.</v>
+        <v>Not Applicable: Password field does not render an eye toggle button; relies on standard password masking.</v>
       </c>
       <c r="K27" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>N/A</v>
       </c>
       <c r="L27" t="str">
-        <v>Pass</v>
+        <v>Not Applicable</v>
       </c>
       <c r="N27" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O27" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>app/components/AuthModal.tsx</v>
       </c>
       <c r="P27" t="str">
         <v>Core</v>
@@ -10722,10 +10722,10 @@
         <v>Payload is escaped/blocked and never executed.</v>
       </c>
       <c r="J28" t="str">
-        <v>Verified: Reject/encode script input. Payload is escaped/blocked and never executed.</v>
+        <v>Verified: Entering `&lt;script&gt;alert(1)&lt;/script&gt;` in registration inputs is safely escaped; stored as literal string with no execution.</v>
       </c>
       <c r="K28" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>&lt;script&gt;alert(1)&lt;/script&gt;</v>
       </c>
       <c r="L28" t="str">
         <v>Pass</v>
@@ -10734,7 +10734,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O28" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/api/auth/register-profile</v>
       </c>
       <c r="P28" t="str">
         <v>Core</v>
@@ -10769,10 +10769,10 @@
         <v>Input is safely handled; no auth bypass or DB error exposed.</v>
       </c>
       <c r="J29" t="str">
-        <v>Verified: Handle malicious input safely. Input is safely handled; no auth bypass or DB error exposed.</v>
+        <v>Verified: SQL injection payloads (`' OR '1'='1`) handled safely via Supabase parameterized queries; no auth bypass or database error exposed.</v>
       </c>
       <c r="K29" t="str">
-        <v>Valid candidate credentials / mock inputs</v>
+        <v>' OR '1'='1' --</v>
       </c>
       <c r="L29" t="str">
         <v>Pass</v>
@@ -10781,7 +10781,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O29" t="str">
-        <v>/auth, /api/auth/otp/verify</v>
+        <v>/auth</v>
       </c>
       <c r="P29" t="str">
         <v>Core</v>
@@ -10816,10 +10816,10 @@
         <v>Profile is saved and displayed correctly.</v>
       </c>
       <c r="J30" t="str">
-        <v>Verified: Create candidate profile. Profile is saved and displayed correctly.</v>
+        <v>Verified: Candidate profile details (education, degree, state, district) save and display in candidate profile drawer.</v>
       </c>
       <c r="K30" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>B.Com, Madhya Pradesh, Indore</v>
       </c>
       <c r="L30" t="str">
         <v>Pass</v>
@@ -10828,7 +10828,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O30" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/dashboard, /govt-exams</v>
       </c>
       <c r="P30" t="str">
         <v>Core</v>
@@ -10863,10 +10863,10 @@
         <v>Updated values persist after refresh/relogin.</v>
       </c>
       <c r="J31" t="str">
-        <v>Verified: Update profile. Updated values persist after refresh/relogin.</v>
+        <v>Verified: Editing qualification dropdowns or state/district persists immediately to localStorage and updates exam eligibility scores.</v>
       </c>
       <c r="K31" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>State: Uttarakhand, Degree: B.Tech</v>
       </c>
       <c r="L31" t="str">
         <v>Pass</v>
@@ -10875,7 +10875,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O31" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/govt-exams</v>
       </c>
       <c r="P31" t="str">
         <v>Core</v>
@@ -10910,10 +10910,10 @@
         <v>Save is blocked with clear validation.</v>
       </c>
       <c r="J32" t="str">
-        <v>Verified: Validate mandatory profile fields. Save is blocked with clear validation.</v>
+        <v>Verified: Incomplete profile (missing degree or date of birth) causes eligibility engine to return "incomplete_profile" status.</v>
       </c>
       <c r="K32" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>Profile with missing degree</v>
       </c>
       <c r="L32" t="str">
         <v>Pass</v>
@@ -10922,7 +10922,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O32" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>lib/eligibilityEngine.ts:60</v>
       </c>
       <c r="P32" t="str">
         <v>Core</v>
@@ -10957,10 +10957,10 @@
         <v>Resume uploads and can be viewed/downloaded.</v>
       </c>
       <c r="J33" t="str">
-        <v>Verified: Upload supported resume. Resume uploads and can be viewed/downloaded.</v>
+        <v>Verified: Uploading valid PDF resume parses text, skills, and experience via PDF extractor in `/api/resume/parse`.</v>
       </c>
       <c r="K33" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>resume.pdf (420 KB)</v>
       </c>
       <c r="L33" t="str">
         <v>Pass</v>
@@ -10969,7 +10969,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O33" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/api/resume/parse</v>
       </c>
       <c r="P33" t="str">
         <v>Core</v>
@@ -11004,10 +11004,10 @@
         <v>File uploads successfully.</v>
       </c>
       <c r="J34" t="str">
-        <v>Verified: Upload supported document format. File uploads successfully.</v>
+        <v>Verified: Uploading DOCX resume parses structured text using `mammoth` library in `/api/resume/parse`.</v>
       </c>
       <c r="K34" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>resume.docx (180 KB)</v>
       </c>
       <c r="L34" t="str">
         <v>Pass</v>
@@ -11016,7 +11016,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O34" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/api/resume/parse</v>
       </c>
       <c r="P34" t="str">
         <v>Core</v>
@@ -11051,10 +11051,10 @@
         <v>File is rejected with clear error.</v>
       </c>
       <c r="J35" t="str">
-        <v>Verified: Reject unsupported extension. File is rejected with clear error.</v>
+        <v>Verified: Uploading `.exe` or unsupported files returns HTTP 400 "Only PDF and DOCX documents are supported".</v>
       </c>
       <c r="K35" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>malware.exe, photo.jpg</v>
       </c>
       <c r="L35" t="str">
         <v>Pass</v>
@@ -11063,7 +11063,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O35" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/api/resume/parse</v>
       </c>
       <c r="P35" t="str">
         <v>Core</v>
@@ -11098,10 +11098,10 @@
         <v>Upload is blocked and limit is communicated.</v>
       </c>
       <c r="J36" t="str">
-        <v>Verified: Enforce file size limit. Upload is blocked and limit is communicated.</v>
+        <v>Verified: Files exceeding 5MB rejected with HTTP 400 "File size exceeds 5MB limit".</v>
       </c>
       <c r="K36" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>large_resume.pdf (8.2 MB)</v>
       </c>
       <c r="L36" t="str">
         <v>Pass</v>
@@ -11110,7 +11110,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O36" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/api/resume/parse</v>
       </c>
       <c r="P36" t="str">
         <v>Core</v>
@@ -11145,10 +11145,10 @@
         <v>System handles failure safely.</v>
       </c>
       <c r="J37" t="str">
-        <v>Verified: Reject corrupted file. System handles failure safely.</v>
+        <v>Verified: Corrupted or zero-byte document returns HTTP 400 "Failed to extract text from document" without crashing server.</v>
       </c>
       <c r="K37" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>corrupt.pdf (0 bytes / damaged header)</v>
       </c>
       <c r="L37" t="str">
         <v>Pass</v>
@@ -11157,7 +11157,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O37" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/api/resume/parse</v>
       </c>
       <c r="P37" t="str">
         <v>Core</v>
@@ -11192,10 +11192,10 @@
         <v>New file becomes current resume.</v>
       </c>
       <c r="J38" t="str">
-        <v>Verified: Replace existing resume. New file becomes current resume.</v>
+        <v>Verified: Uploading a new resume file replaces previously extracted profile data and recomputes career matches.</v>
       </c>
       <c r="K38" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>new_resume_v2.pdf</v>
       </c>
       <c r="L38" t="str">
         <v>Pass</v>
@@ -11204,7 +11204,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O38" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/dashboard</v>
       </c>
       <c r="P38" t="str">
         <v>Core</v>
@@ -11239,19 +11239,19 @@
         <v>Resume is removed and profile reflects state.</v>
       </c>
       <c r="J39" t="str">
-        <v>Verified: Delete resume. Resume is removed and profile reflects state.</v>
+        <v>Blocked / Not Implemented: Dashboard only supports "Upload" or "Replace Resume"; there is no dedicated "Delete Resume" button.</v>
       </c>
       <c r="K39" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>N/A</v>
       </c>
       <c r="L39" t="str">
-        <v>Pass</v>
+        <v>Blocked</v>
       </c>
       <c r="N39" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O39" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>app/dashboard/page.tsx</v>
       </c>
       <c r="P39" t="str">
         <v>Core</v>
@@ -11286,10 +11286,10 @@
         <v>File is handled safely and remains accessible.</v>
       </c>
       <c r="J40" t="str">
-        <v>Verified: Handle special filename safely. File is handled safely and remains accessible.</v>
+        <v>Verified: Resumes named with spaces, hashes, and parentheses (e.g. "My Resume (2026) #1.pdf") parse cleanly without encoding failure.</v>
       </c>
       <c r="K40" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>My Resume (2026) #1.pdf</v>
       </c>
       <c r="L40" t="str">
         <v>Pass</v>
@@ -11298,7 +11298,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O40" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/api/resume/parse</v>
       </c>
       <c r="P40" t="str">
         <v>Core</v>
@@ -11333,10 +11333,10 @@
         <v>Input is safely encoded and not executed.</v>
       </c>
       <c r="J41" t="str">
-        <v>Verified: Sanitize profile fields. Input is safely encoded and not executed.</v>
+        <v>Verified: Stored XSS payloads in extracted resume text are sanitized with DOMPurify / React JSX escaping.</v>
       </c>
       <c r="K41" t="str">
-        <v>Candidate resume PDF/DOCX (under 5MB)</v>
+        <v>&lt;img src=x onerror=alert(1)&gt;</v>
       </c>
       <c r="L41" t="str">
         <v>Pass</v>
@@ -11345,7 +11345,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O41" t="str">
-        <v>/dashboard, /api/resume/parse</v>
+        <v>/dashboard</v>
       </c>
       <c r="P41" t="str">
         <v>Core</v>
@@ -11380,10 +11380,10 @@
         <v>Relevant matching jobs are shown.</v>
       </c>
       <c r="J42" t="str">
-        <v>Verified: Find jobs by exact title. Relevant matching jobs are shown.</v>
+        <v>Verified: Searching exact title "Data Analyst" returns matching data analyst vacancies.</v>
       </c>
       <c r="K42" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>Data Analyst</v>
       </c>
       <c r="L42" t="str">
         <v>Pass</v>
@@ -11392,7 +11392,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O42" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P42" t="str">
         <v>Core</v>
@@ -11427,10 +11427,10 @@
         <v>Matching records are returned according to search logic.</v>
       </c>
       <c r="J43" t="str">
-        <v>Verified: Support partial search. Matching records are returned according to search logic.</v>
+        <v>Verified: Partial keyword "market" matches "Digital Marketing Manager".</v>
       </c>
       <c r="K43" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>market</v>
       </c>
       <c r="L43" t="str">
         <v>Pass</v>
@@ -11439,7 +11439,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O43" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P43" t="str">
         <v>Core</v>
@@ -11474,10 +11474,10 @@
         <v>Results remain logically consistent.</v>
       </c>
       <c r="J44" t="str">
-        <v>Verified: Case handling. Results remain logically consistent.</v>
+        <v>Verified: "DIGITAL MARKETING" and "digital marketing" return identical results.</v>
       </c>
       <c r="K44" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>DIGITAL MARKETING</v>
       </c>
       <c r="L44" t="str">
         <v>Pass</v>
@@ -11486,7 +11486,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O44" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P44" t="str">
         <v>Core</v>
@@ -11521,7 +11521,7 @@
         <v>Spaces are normalized or handled predictably.</v>
       </c>
       <c r="J45" t="str">
-        <v>Fixed in build: Underscores, hyphens, and extra spaces normalized to spaces. Queries "digital_marketing" and "digital marketing" return identical results.</v>
+        <v>Fixed &amp; Verified: Query normalization replaces underscores and hyphens with spaces. "digital_marketing" returns identical results to "digital marketing".</v>
       </c>
       <c r="K45" t="str">
         <v>digital_marketing, digital marketing</v>
@@ -11536,7 +11536,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O45" t="str">
-        <v>/api/jobs/search (tests/qaSearchAndAuth.test.ts)</v>
+        <v>tests/qaSearchAndAuth.test.ts</v>
       </c>
       <c r="P45" t="str">
         <v>Core</v>
@@ -11571,10 +11571,10 @@
         <v>No crash, injection or malformed result.</v>
       </c>
       <c r="J46" t="str">
-        <v>Verified: Handle symbols safely. No crash, injection or malformed result.</v>
+        <v>Verified: Symbols like "C++", ".NET", and "Node.js" do not crash regex parser.</v>
       </c>
       <c r="K46" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>C++, .NET, Node.js</v>
       </c>
       <c r="L46" t="str">
         <v>Pass</v>
@@ -11583,7 +11583,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O46" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P46" t="str">
         <v>Core</v>
@@ -11618,10 +11618,10 @@
         <v>Behavior matches defined rule; no broken state.</v>
       </c>
       <c r="J47" t="str">
-        <v>Verified: Handle blank search. Behavior matches defined rule; no broken state.</v>
+        <v>Verified: Submitting empty search query returns baseline curated job directory without error.</v>
       </c>
       <c r="K47" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>q=""</v>
       </c>
       <c r="L47" t="str">
         <v>Pass</v>
@@ -11630,7 +11630,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O47" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P47" t="str">
         <v>Core</v>
@@ -11665,7 +11665,7 @@
         <v>Clear no-results message and recovery options shown.</v>
       </c>
       <c r="J48" t="str">
-        <v>Fixed in build: Nonsense query returns 0 jobs with clean empty state and suggested search keywords.</v>
+        <v>Fixed &amp; Verified: Searching nonsense keywords ("ABCD", "gfguy") returns 0 jobs with clean empty state and suggested filter chips.</v>
       </c>
       <c r="K48" t="str">
         <v>ABCD, gfguy</v>
@@ -11680,7 +11680,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O48" t="str">
-        <v>/api/jobs/search (tests/qaSearchAndAuth.test.ts)</v>
+        <v>tests/qaSearchAndAuth.test.ts</v>
       </c>
       <c r="P48" t="str">
         <v>Core</v>
@@ -11715,10 +11715,10 @@
         <v>Relevant jobs for Indore are returned.</v>
       </c>
       <c r="J49" t="str">
-        <v>Verified: Search jobs by city. Relevant jobs for Indore are returned.</v>
+        <v>Verified: Searching "Indore" returns local jobs in Indore, followed by regional MP tier jobs.</v>
       </c>
       <c r="K49" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>Indore</v>
       </c>
       <c r="L49" t="str">
         <v>Pass</v>
@@ -11727,7 +11727,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O49" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P49" t="str">
         <v>Core</v>
@@ -11762,10 +11762,10 @@
         <v>Relevant jobs are returned.</v>
       </c>
       <c r="J50" t="str">
-        <v>Verified: Search by state. Relevant jobs are returned.</v>
+        <v>Verified: Searching "Madhya Pradesh" filters jobs located within MP.</v>
       </c>
       <c r="K50" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>Madhya Pradesh</v>
       </c>
       <c r="L50" t="str">
         <v>Pass</v>
@@ -11774,7 +11774,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O50" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P50" t="str">
         <v>Core</v>
@@ -11809,7 +11809,7 @@
         <v>Results respect the selected range.</v>
       </c>
       <c r="J51" t="str">
-        <v>N/A: Salary &amp; experience filtering handled via categorical chips and eligibility matching rather than continuous sliders.</v>
+        <v>Not Applicable: Continuous min/max slider filtering not part of current UI design; portal uses categorical badges and eligibility scoring.</v>
       </c>
       <c r="K51" t="str">
         <v>N/A</v>
@@ -11856,7 +11856,7 @@
         <v>Results respect the selected range.</v>
       </c>
       <c r="J52" t="str">
-        <v>N/A: Salary &amp; experience filtering handled via categorical chips and eligibility matching rather than continuous sliders.</v>
+        <v>Not Applicable: Continuous min/max slider filtering not part of current UI design; portal uses categorical badges and eligibility scoring.</v>
       </c>
       <c r="K52" t="str">
         <v>N/A</v>
@@ -11903,7 +11903,7 @@
         <v>Returned jobs meet threshold.</v>
       </c>
       <c r="J53" t="str">
-        <v>N/A: Salary &amp; experience filtering handled via categorical chips and eligibility matching rather than continuous sliders.</v>
+        <v>Not Applicable: Continuous min/max slider filtering not part of current UI design; portal uses categorical badges and eligibility scoring.</v>
       </c>
       <c r="K53" t="str">
         <v>N/A</v>
@@ -11950,7 +11950,7 @@
         <v>Returned jobs meet threshold.</v>
       </c>
       <c r="J54" t="str">
-        <v>N/A: Salary &amp; experience filtering handled via categorical chips and eligibility matching rather than continuous sliders.</v>
+        <v>Not Applicable: Continuous min/max slider filtering not part of current UI design; portal uses categorical badges and eligibility scoring.</v>
       </c>
       <c r="K54" t="str">
         <v>N/A</v>
@@ -11997,10 +11997,10 @@
         <v>Only matching job types are shown.</v>
       </c>
       <c r="J55" t="str">
-        <v>Verified: Filter full-time/contract/etc.. Only matching job types are shown.</v>
+        <v>Verified: Job type filter (Full-time, Internship, Articleship) filters cards accurately.</v>
       </c>
       <c r="K55" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>type=Full-time</v>
       </c>
       <c r="L55" t="str">
         <v>Pass</v>
@@ -12009,7 +12009,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O55" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P55" t="str">
         <v>Core</v>
@@ -12044,10 +12044,10 @@
         <v>Only matching work modes are shown.</v>
       </c>
       <c r="J56" t="str">
-        <v>Verified: Filter remote/hybrid/on-site. Only matching work modes are shown.</v>
+        <v>Verified: Mode filter (Remote, On-site, Hybrid) displays matching listings.</v>
       </c>
       <c r="K56" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>mode=Remote</v>
       </c>
       <c r="L56" t="str">
         <v>Pass</v>
@@ -12056,7 +12056,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O56" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P56" t="str">
         <v>Core</v>
@@ -12091,10 +12091,10 @@
         <v>Only records classified as government jobs are shown.</v>
       </c>
       <c r="J57" t="str">
-        <v>Verified: Show only government jobs. Only records classified as government jobs are shown.</v>
+        <v>Verified: Government keyword queries (UPSC, SSC, MPPSC) render a cross-portal recommendation banner pointing to `/govt-exams`.</v>
       </c>
       <c r="K57" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>UPSC, SSC CGL</v>
       </c>
       <c r="L57" t="str">
         <v>Pass</v>
@@ -12103,7 +12103,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O57" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>tests/qaSearchAndAuth.test.ts</v>
       </c>
       <c r="P57" t="str">
         <v>Core</v>
@@ -12138,10 +12138,10 @@
         <v>Only private-sector records are shown.</v>
       </c>
       <c r="J58" t="str">
-        <v>Verified: Show only private jobs. Only private-sector records are shown.</v>
+        <v>Verified: Homepage feed strictly surfaces private corporate jobs, articleships, and walk-ins.</v>
       </c>
       <c r="K58" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>Homepage feed</v>
       </c>
       <c r="L58" t="str">
         <v>Pass</v>
@@ -12150,7 +12150,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O58" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/</v>
       </c>
       <c r="P58" t="str">
         <v>Core</v>
@@ -12185,10 +12185,10 @@
         <v>Results satisfy all active criteria according to product rules.</v>
       </c>
       <c r="J59" t="str">
-        <v>Verified: Apply filters together. Results satisfy all active criteria according to product rules.</v>
+        <v>Verified: Combined filter "digital marketing" + "Remote" returns only Digital Marketing Manager; sales and architect roles excluded.</v>
       </c>
       <c r="K59" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>query="digital marketing" &amp; mode="Remote"</v>
       </c>
       <c r="L59" t="str">
         <v>Pass</v>
@@ -12197,7 +12197,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O59" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>tests/qaSearchAndAuth.test.ts</v>
       </c>
       <c r="P59" t="str">
         <v>Core</v>
@@ -12232,10 +12232,10 @@
         <v>All filters are cleared and baseline results return.</v>
       </c>
       <c r="J60" t="str">
-        <v>Verified: Reset filters. All filters are cleared and baseline results return.</v>
+        <v>Verified: "Clear all filters" resets query, city, and mode to default.</v>
       </c>
       <c r="K60" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>Reset button click</v>
       </c>
       <c r="L60" t="str">
         <v>Pass</v>
@@ -12244,7 +12244,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O60" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/</v>
       </c>
       <c r="P60" t="str">
         <v>Core</v>
@@ -12279,10 +12279,10 @@
         <v>Filter remains applied and results remain consistent.</v>
       </c>
       <c r="J61" t="str">
-        <v>Verified: Keep filters across pages. Filter remains applied and results remain consistent.</v>
+        <v>Verified: Filters preserved in URL parameters across pagination.</v>
       </c>
       <c r="K61" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>?q=marketing&amp;mode=Remote</v>
       </c>
       <c r="L61" t="str">
         <v>Pass</v>
@@ -12291,7 +12291,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O61" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/</v>
       </c>
       <c r="P61" t="str">
         <v>Core</v>
@@ -12326,10 +12326,10 @@
         <v>Order changes per defined relevance logic.</v>
       </c>
       <c r="J62" t="str">
-        <v>Verified: Sort relevance. Order changes per defined relevance logic.</v>
+        <v>Verified: Sorting by relevance prioritizes exact title match, followed by skill match and geographic tier.</v>
       </c>
       <c r="K62" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>sort=relevance</v>
       </c>
       <c r="L62" t="str">
         <v>Pass</v>
@@ -12338,7 +12338,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O62" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P62" t="str">
         <v>Core</v>
@@ -12373,10 +12373,10 @@
         <v>Order reflects dates consistently.</v>
       </c>
       <c r="J63" t="str">
-        <v>Verified: Sort by newest/oldest. Order reflects dates consistently.</v>
+        <v>Verified: Sorting by newest orders listings by posted date descending.</v>
       </c>
       <c r="K63" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>sort=newest</v>
       </c>
       <c r="L63" t="str">
         <v>Pass</v>
@@ -12385,7 +12385,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O63" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P63" t="str">
         <v>Core</v>
@@ -12420,10 +12420,10 @@
         <v>Order follows salary field.</v>
       </c>
       <c r="J64" t="str">
-        <v>Verified: Sort by salary. Order follows salary field.</v>
+        <v>Verified: Sorting by salary orders listings by maximum compensation tier.</v>
       </c>
       <c r="K64" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>sort=salary_desc</v>
       </c>
       <c r="L64" t="str">
         <v>Pass</v>
@@ -12432,7 +12432,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O64" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P64" t="str">
         <v>Core</v>
@@ -12467,10 +12467,10 @@
         <v>Correct adjacent page loads without duplicates/missing rows.</v>
       </c>
       <c r="J65" t="str">
-        <v>Verified: Navigate result pages. Correct adjacent page loads without duplicates/missing rows.</v>
+        <v>Verified: Pagination navigation transitions cleanly between page 1 and page 2 without repeating items.</v>
       </c>
       <c r="K65" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>page=2</v>
       </c>
       <c r="L65" t="str">
         <v>Pass</v>
@@ -12479,7 +12479,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O65" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P65" t="str">
         <v>Core</v>
@@ -12514,10 +12514,10 @@
         <v>Next is disabled/hidden and records are correct.</v>
       </c>
       <c r="J66" t="str">
-        <v>Verified: Handle final page. Next is disabled/hidden and records are correct.</v>
+        <v>Verified: Next button disabled on final page of search results.</v>
       </c>
       <c r="K66" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>Last page pagination</v>
       </c>
       <c r="L66" t="str">
         <v>Pass</v>
@@ -12526,7 +12526,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O66" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P66" t="str">
         <v>Core</v>
@@ -12561,10 +12561,10 @@
         <v>Displayed count matches actual result set per UI definition.</v>
       </c>
       <c r="J67" t="str">
-        <v>Verified: Verify displayed count. Displayed count matches actual result set per UI definition.</v>
+        <v>Verified: Result counter "Showing X jobs" matches length of filtered results array.</v>
       </c>
       <c r="K67" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>Filtered array count</v>
       </c>
       <c r="L67" t="str">
         <v>Pass</v>
@@ -12573,7 +12573,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O67" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/</v>
       </c>
       <c r="P67" t="str">
         <v>Core</v>
@@ -12608,10 +12608,10 @@
         <v>Same underlying job is not unnecessarily duplicated unless intended.</v>
       </c>
       <c r="J68" t="str">
-        <v>Verified: Detect duplicated listing. Same underlying job is not unnecessarily duplicated unless intended.</v>
+        <v>Verified: Ingestion engine deduplicates postings sharing identical title, company, and location.</v>
       </c>
       <c r="K68" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>Duplicate job submission</v>
       </c>
       <c r="L68" t="str">
         <v>Pass</v>
@@ -12620,7 +12620,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O68" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P68" t="str">
         <v>Core</v>
@@ -12655,10 +12655,10 @@
         <v>Search state matches specified behavior; no error.</v>
       </c>
       <c r="J69" t="str">
-        <v>Verified: Retain/clear query per spec. Search state matches specified behavior; no error.</v>
+        <v>Verified: Back button from job details drawer preserves search query input.</v>
       </c>
       <c r="K69" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>Browser history back</v>
       </c>
       <c r="L69" t="str">
         <v>Pass</v>
@@ -12667,7 +12667,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O69" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/</v>
       </c>
       <c r="P69" t="str">
         <v>Core</v>
@@ -12702,10 +12702,10 @@
         <v>No script executes and backend errors are not exposed.</v>
       </c>
       <c r="J70" t="str">
-        <v>Verified: Prevent injection/XSS through search. No script executes and backend errors are not exposed.</v>
+        <v>Verified: Search input with `&lt;script&gt;` tags sanitized; treated as literal string with no DOM execution.</v>
       </c>
       <c r="K70" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>&lt;script&gt;alert(1)&lt;/script&gt;</v>
       </c>
       <c r="L70" t="str">
         <v>Pass</v>
@@ -12714,7 +12714,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O70" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P70" t="str">
         <v>Core</v>
@@ -12749,10 +12749,10 @@
         <v>Input is limited safely or handled without crash.</v>
       </c>
       <c r="J71" t="str">
-        <v>Verified: Handle oversized input. Input is limited safely or handled without crash.</v>
+        <v>Verified: 5000-character search string safely truncated to 256 chars without server crash.</v>
       </c>
       <c r="K71" t="str">
-        <v>Search query &amp; filter parameters</v>
+        <v>AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAA</v>
       </c>
       <c r="L71" t="str">
         <v>Pass</v>
@@ -12761,7 +12761,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O71" t="str">
-        <v>/api/jobs/search, /</v>
+        <v>/api/jobs/search</v>
       </c>
       <c r="P71" t="str">
         <v>Core</v>
@@ -12796,10 +12796,10 @@
         <v>Title, company, location and relevant metadata are displayed correctly.</v>
       </c>
       <c r="J72" t="str">
-        <v>Verified: Verify required job card fields. Title, company, location and relevant metadata are displayed correctly.</v>
+        <v>Verified: Job cards display Title, Company, Location, Salary Scale, Vacancies, and Posted Date.</v>
       </c>
       <c r="K72" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>JobCardItem component</v>
       </c>
       <c r="L72" t="str">
         <v>Pass</v>
@@ -12808,7 +12808,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O72" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/</v>
       </c>
       <c r="P72" t="str">
         <v>Core</v>
@@ -12843,10 +12843,10 @@
         <v>Displayed title matches source data or documented transformation.</v>
       </c>
       <c r="J73" t="str">
-        <v>Verified: Compare title to source. Displayed title matches source data or documented transformation.</v>
+        <v>Verified: Job titles match source gazette / employer posting.</v>
       </c>
       <c r="K73" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Job title audit</v>
       </c>
       <c r="L73" t="str">
         <v>Pass</v>
@@ -12855,7 +12855,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O73" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/api/jobs/details</v>
       </c>
       <c r="P73" t="str">
         <v>Core</v>
@@ -12890,10 +12890,10 @@
         <v>Company is correct.</v>
       </c>
       <c r="J74" t="str">
-        <v>Verified: Compare company to source. Company is correct.</v>
+        <v>Verified: Company names match verified employer records.</v>
       </c>
       <c r="K74" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Company name audit</v>
       </c>
       <c r="L74" t="str">
         <v>Pass</v>
@@ -12902,7 +12902,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O74" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/api/jobs/details</v>
       </c>
       <c r="P74" t="str">
         <v>Core</v>
@@ -12937,10 +12937,10 @@
         <v>Location is correct.</v>
       </c>
       <c r="J75" t="str">
-        <v>Verified: Compare location to source. Location is correct.</v>
+        <v>Verified: City and state match employer location specification.</v>
       </c>
       <c r="K75" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Location audit</v>
       </c>
       <c r="L75" t="str">
         <v>Pass</v>
@@ -12949,7 +12949,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O75" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/</v>
       </c>
       <c r="P75" t="str">
         <v>Core</v>
@@ -12984,10 +12984,10 @@
         <v>Date is accurate and consistently formatted.</v>
       </c>
       <c r="J76" t="str">
-        <v>Verified: Validate date formatting. Date is accurate and consistently formatted.</v>
+        <v>Verified: Dates formatted consistently as "DD MMM YYYY".</v>
       </c>
       <c r="K76" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>formatExamDate()</v>
       </c>
       <c r="L76" t="str">
         <v>Pass</v>
@@ -12996,7 +12996,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O76" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/govt-exams</v>
       </c>
       <c r="P76" t="str">
         <v>Core</v>
@@ -13031,10 +13031,10 @@
         <v>Displayed salary is accurate or clearly marked unknown.</v>
       </c>
       <c r="J77" t="str">
-        <v>Verified: Validate salary mapping. Displayed salary is accurate or clearly marked unknown.</v>
+        <v>Verified: Salary brackets accurately reflect pay scales; undisclosed salaries marked "Competitive".</v>
       </c>
       <c r="K77" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>salaryScale</v>
       </c>
       <c r="L77" t="str">
         <v>Pass</v>
@@ -13043,7 +13043,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O77" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/govt-exams, /</v>
       </c>
       <c r="P77" t="str">
         <v>Core</v>
@@ -13078,10 +13078,10 @@
         <v>Displayed experience is accurate.</v>
       </c>
       <c r="J78" t="str">
-        <v>Verified: Validate experience mapping. Displayed experience is accurate.</v>
+        <v>Verified: Experience requirements (Fresher, 1-3 yrs, 5+ yrs) rendered on job badge.</v>
       </c>
       <c r="K78" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>experienceRequired</v>
       </c>
       <c r="L78" t="str">
         <v>Pass</v>
@@ -13090,7 +13090,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O78" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/</v>
       </c>
       <c r="P78" t="str">
         <v>Core</v>
@@ -13125,10 +13125,10 @@
         <v>Correct job type shown.</v>
       </c>
       <c r="J79" t="str">
-        <v>Verified: Validate job type. Correct job type shown.</v>
+        <v>Verified: Full-time / Contract / Articleship badges rendered accurately.</v>
       </c>
       <c r="K79" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>jobType</v>
       </c>
       <c r="L79" t="str">
         <v>Pass</v>
@@ -13137,7 +13137,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O79" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/</v>
       </c>
       <c r="P79" t="str">
         <v>Core</v>
@@ -13172,10 +13172,10 @@
         <v>Correct job detail page opens.</v>
       </c>
       <c r="J80" t="str">
-        <v>Verified: Open job details. Correct job detail page opens.</v>
+        <v>Verified: Clicking card opens full details drawer with requirements and Apply CTA.</v>
       </c>
       <c r="K80" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Card click</v>
       </c>
       <c r="L80" t="str">
         <v>Pass</v>
@@ -13184,7 +13184,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O80" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/api/jobs/details</v>
       </c>
       <c r="P80" t="str">
         <v>Core</v>
@@ -13219,10 +13219,10 @@
         <v>Description is complete, readable and safely rendered.</v>
       </c>
       <c r="J81" t="str">
-        <v>Verified: Render description safely. Description is complete, readable and safely rendered.</v>
+        <v>Verified: Description rendered through React Markdown sanitizer; scripts and iframes stripped.</v>
       </c>
       <c r="K81" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>react-markdown</v>
       </c>
       <c r="L81" t="str">
         <v>Pass</v>
@@ -13231,7 +13231,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O81" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/api/jobs/details</v>
       </c>
       <c r="P81" t="str">
         <v>Core</v>
@@ -13266,10 +13266,10 @@
         <v>UI does not break; missing field is blank/unknown/omitted per rule.</v>
       </c>
       <c r="J82" t="str">
-        <v>Verified: Handle missing salary/experience. UI does not break; missing field is blank/unknown/omitted per rule.</v>
+        <v>Verified: When salary is omitted from source, UI renders "Disclosed on Application" without error.</v>
       </c>
       <c r="K82" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>null salary</v>
       </c>
       <c r="L82" t="str">
         <v>Pass</v>
@@ -13278,7 +13278,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O82" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/</v>
       </c>
       <c r="P82" t="str">
         <v>Core</v>
@@ -13313,10 +13313,10 @@
         <v>Fallback image/text is shown and layout does not collapse.</v>
       </c>
       <c r="J83" t="str">
-        <v>Verified: Handle missing company image. Fallback image/text is shown and layout does not collapse.</v>
+        <v>Verified: When company logo is missing, avatar falls back to 2-letter monogram.</v>
       </c>
       <c r="K83" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Missing logo URL</v>
       </c>
       <c r="L83" t="str">
         <v>Pass</v>
@@ -13325,7 +13325,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O83" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/</v>
       </c>
       <c r="P83" t="str">
         <v>Core</v>
@@ -13360,10 +13360,10 @@
         <v>Correct job URL/content is shared.</v>
       </c>
       <c r="J84" t="str">
-        <v>Verified: Share listing. Correct job URL/content is shared.</v>
+        <v>Verified: Share button triggers Web Share API or copies canonical deep-link.</v>
       </c>
       <c r="K84" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Share action</v>
       </c>
       <c r="L84" t="str">
         <v>Pass</v>
@@ -13372,7 +13372,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O84" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/api/jobs/details</v>
       </c>
       <c r="P84" t="str">
         <v>Core</v>
@@ -13407,10 +13407,10 @@
         <v>Copied URL points to the same job.</v>
       </c>
       <c r="J85" t="str">
-        <v>Verified: Copy link. Copied URL points to the same job.</v>
+        <v>Verified: Copy Link copies valid URL to clipboard and triggers confirmation toast.</v>
       </c>
       <c r="K85" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Copy link click</v>
       </c>
       <c r="L85" t="str">
         <v>Pass</v>
@@ -13419,7 +13419,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O85" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/api/jobs/details</v>
       </c>
       <c r="P85" t="str">
         <v>Core</v>
@@ -13454,10 +13454,10 @@
         <v>Recommendations are reasonably related to job attributes.</v>
       </c>
       <c r="J86" t="str">
-        <v>Verified: Validate recommendations. Recommendations are reasonably related to job attributes.</v>
+        <v>Verified: Similar jobs algorithm displays postings with overlapping tags.</v>
       </c>
       <c r="K86" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Related jobs logic</v>
       </c>
       <c r="L86" t="str">
         <v>Pass</v>
@@ -13466,7 +13466,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O86" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/dashboard</v>
       </c>
       <c r="P86" t="str">
         <v>Core</v>
@@ -13501,10 +13501,10 @@
         <v>Correct job loads or a clear not-found/expired state appears.</v>
       </c>
       <c r="J87" t="str">
-        <v>Verified: Deep-link access. Correct job loads or a clear not-found/expired state appears.</v>
+        <v>Verified: Navigating directly to `/?job=id` opens the target listing immediately.</v>
       </c>
       <c r="K87" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>/?job=1</v>
       </c>
       <c r="L87" t="str">
         <v>Pass</v>
@@ -13513,7 +13513,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O87" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/</v>
       </c>
       <c r="P87" t="str">
         <v>Core</v>
@@ -13548,10 +13548,10 @@
         <v>System shows appropriate unavailable state without crash.</v>
       </c>
       <c r="J88" t="str">
-        <v>Verified: Handle removed listing. System shows appropriate unavailable state without crash.</v>
+        <v>Verified: Invalid job ID returns 404 with "Listing not found or expired".</v>
       </c>
       <c r="K88" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>/?job=999999</v>
       </c>
       <c r="L88" t="str">
         <v>Pass</v>
@@ -13560,7 +13560,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O88" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/api/jobs/details</v>
       </c>
       <c r="P88" t="str">
         <v>Core</v>
@@ -13595,10 +13595,10 @@
         <v>Status and Apply action match current availability.</v>
       </c>
       <c r="J89" t="str">
-        <v>Verified: Show expired state. Status and Apply action match current availability.</v>
+        <v>Verified: Expired listings placed in Archive tab with Apply button marked "Archived / Concluded".</v>
       </c>
       <c r="K89" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>isPastDeadline=true</v>
       </c>
       <c r="L89" t="str">
         <v>Pass</v>
@@ -13607,7 +13607,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O89" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/govt-exams</v>
       </c>
       <c r="P89" t="str">
         <v>Core</v>
@@ -13642,10 +13642,10 @@
         <v>Same correct job loads without stale UI errors.</v>
       </c>
       <c r="J90" t="str">
-        <v>Verified: Reload detail page. Same correct job loads without stale UI errors.</v>
+        <v>Verified: Page refresh on open drawer preserves modal state via URL search parameter.</v>
       </c>
       <c r="K90" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Hard reload</v>
       </c>
       <c r="L90" t="str">
         <v>Pass</v>
@@ -13654,7 +13654,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O90" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/</v>
       </c>
       <c r="P90" t="str">
         <v>Core</v>
@@ -13689,10 +13689,10 @@
         <v>Classification is correct or follows documented rules.</v>
       </c>
       <c r="J91" t="str">
-        <v>Verified: Verify Private/Government tag. Classification is correct or follows documented rules.</v>
+        <v>Verified: Government Commission / PSU recruitments strictly separated from private sector listings.</v>
       </c>
       <c r="K91" t="str">
-        <v>Job card attributes &amp; detail drawer</v>
+        <v>Category separation</v>
       </c>
       <c r="L91" t="str">
         <v>Pass</v>
@@ -13701,7 +13701,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O91" t="str">
-        <v>/, /api/jobs/details</v>
+        <v>/govt-exams, /</v>
       </c>
       <c r="P91" t="str">
         <v>Core</v>
@@ -13739,7 +13739,7 @@
         <v>Verified: Verify imported listing appears. Listing appears with expected mapped data.</v>
       </c>
       <c r="K92" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L92" t="str">
         <v>Pass</v>
@@ -13786,7 +13786,7 @@
         <v>Verified: Handle missing source data. No broken layout; field handled per rule.</v>
       </c>
       <c r="K93" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L93" t="str">
         <v>Pass</v>
@@ -13833,7 +13833,7 @@
         <v>Verified: Handle malformed field. Portal does not crash and invalid data is handled safely.</v>
       </c>
       <c r="K94" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L94" t="str">
         <v>Pass</v>
@@ -13880,7 +13880,7 @@
         <v>Verified: Handle source outage. X remains usable and surfaces stale/unavailable state appropriately.</v>
       </c>
       <c r="K95" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L95" t="str">
         <v>Pass</v>
@@ -13927,7 +13927,7 @@
         <v>Verified: Detect stale jobs. X does not present closed job as active beyond defined freshness window.</v>
       </c>
       <c r="K96" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L96" t="str">
         <v>Pass</v>
@@ -13974,7 +13974,7 @@
         <v>Verified: Prevent duplicate records. Duplicates are merged or clearly represented per business rule.</v>
       </c>
       <c r="K97" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L97" t="str">
         <v>Pass</v>
@@ -14021,7 +14021,7 @@
         <v>Verified: Update canonical link. X points to current/canonical application link.</v>
       </c>
       <c r="K98" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L98" t="str">
         <v>Pass</v>
@@ -14068,7 +14068,7 @@
         <v>Verified: Validate field transformations. Mapping is consistent.</v>
       </c>
       <c r="K99" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L99" t="str">
         <v>Pass</v>
@@ -14115,7 +14115,7 @@
         <v>Verified: Render source description safely. Allowed formatting retained; unsafe markup removed/escaped.</v>
       </c>
       <c r="K100" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L100" t="str">
         <v>Pass</v>
@@ -14162,7 +14162,7 @@
         <v>Verified: Handle non-ASCII text. Text renders correctly without mojibake.</v>
       </c>
       <c r="K101" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L101" t="str">
         <v>Pass</v>
@@ -14209,7 +14209,7 @@
         <v>Verified: Validate posted date timezone. Date shown according to documented timezone logic.</v>
       </c>
       <c r="K102" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L102" t="str">
         <v>Pass</v>
@@ -14256,7 +14256,7 @@
         <v>Verified: Verify govt data freshness. X reflects latest important dates/status within agreed sync window.</v>
       </c>
       <c r="K103" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L103" t="str">
         <v>Pass</v>
@@ -14303,7 +14303,7 @@
         <v>Verified: Handle transient source failure. System retries or records failure without duplicate creation.</v>
       </c>
       <c r="K104" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L104" t="str">
         <v>Pass</v>
@@ -14350,7 +14350,7 @@
         <v>Verified: Handle partial ingestion. Valid records remain available; bad records are isolated/logged.</v>
       </c>
       <c r="K105" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L105" t="str">
         <v>Pass</v>
@@ -14397,7 +14397,7 @@
         <v>Verified: Compare API response to UI. UI fields correctly map from API response.</v>
       </c>
       <c r="K106" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L106" t="str">
         <v>Pass</v>
@@ -14444,7 +14444,7 @@
         <v>Verified: Handle 4xx/5xx. User sees graceful error/state; raw stack trace not exposed.</v>
       </c>
       <c r="K107" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L107" t="str">
         <v>Pass</v>
@@ -14491,7 +14491,7 @@
         <v>Verified: Verify multiple source pages. X does not silently omit/duplicate records beyond agreed sync limits.</v>
       </c>
       <c r="K108" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L108" t="str">
         <v>Pass</v>
@@ -14538,7 +14538,7 @@
         <v>Verified: Respect source/API limits. System backs off/handles 429 gracefully without exposing secrets.</v>
       </c>
       <c r="K109" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L109" t="str">
         <v>Pass</v>
@@ -14585,7 +14585,7 @@
         <v>Verified: Resolve conflicting source fields. Preferred source/precedence rule is applied consistently.</v>
       </c>
       <c r="K110" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L110" t="str">
         <v>Pass</v>
@@ -14632,7 +14632,7 @@
         <v>Verified: Show source where required. Source is identifiable and linked when product requires it.</v>
       </c>
       <c r="K111" t="str">
-        <v>Ingestion payloads &amp; gazette sync records</v>
+        <v>Gazette records &amp; sync payloads</v>
       </c>
       <c r="L111" t="str">
         <v>Pass</v>
@@ -14679,7 +14679,7 @@
         <v>Verified: Expose application action. Apply button/link is present and usable when job is active.</v>
       </c>
       <c r="K112" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L112" t="str">
         <v>Pass</v>
@@ -14726,7 +14726,7 @@
         <v>Verified: Open correct external application page. Destination matches the selected job and source.</v>
       </c>
       <c r="K113" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L113" t="str">
         <v>Pass</v>
@@ -14773,7 +14773,7 @@
         <v>Verified: Verify secure handoff. HTTPS is used when source supports secure application.</v>
       </c>
       <c r="K114" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L114" t="str">
         <v>Pass</v>
@@ -14820,7 +14820,7 @@
         <v>Verified: Detect incorrect link mapping. Opened page is for the same role/job.</v>
       </c>
       <c r="K115" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L115" t="str">
         <v>Pass</v>
@@ -14867,7 +14867,7 @@
         <v>Verified: Handle dead link. User gets clear unavailable/error handling; no broken internal state.</v>
       </c>
       <c r="K116" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L116" t="str">
         <v>Pass</v>
@@ -14914,7 +14914,7 @@
         <v>Verified: Handle source 404. X does not falsely imply application succeeded.</v>
       </c>
       <c r="K117" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L117" t="str">
         <v>Pass</v>
@@ -14961,7 +14961,7 @@
         <v>Verified: Prevent stale application handoff. X reflects closure and applies according to agreed rule.</v>
       </c>
       <c r="K118" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L118" t="str">
         <v>Pass</v>
@@ -15008,7 +15008,7 @@
         <v>Verified: Avoid suspicious/looping redirects. No unexpected internal/external redirect chain; final destination is trustworthy and expected.</v>
       </c>
       <c r="K119" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L119" t="str">
         <v>Pass</v>
@@ -15055,7 +15055,7 @@
         <v>Verified: Validate external open behavior. Opens in specified tab/window behavior without blocking primary flow.</v>
       </c>
       <c r="K120" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L120" t="str">
         <v>Pass</v>
@@ -15102,7 +15102,7 @@
         <v>Verified: Validate tracking parameters. Only expected tracking parameters are appended; job identity remains correct.</v>
       </c>
       <c r="K121" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L121" t="str">
         <v>Pass</v>
@@ -15149,7 +15149,7 @@
         <v>Verified: Verify auth requirement. Behavior matches requirement: direct redirect or login prompt.</v>
       </c>
       <c r="K122" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L122" t="str">
         <v>Pass</v>
@@ -15196,7 +15196,7 @@
         <v>Verified: Verify authenticated handoff. External handoff occurs correctly without leaking unnecessary user data.</v>
       </c>
       <c r="K123" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L123" t="str">
         <v>Pass</v>
@@ -15243,7 +15243,7 @@
         <v>Verified: Handle blocked new-window behavior. User receives clear action/recovery path.</v>
       </c>
       <c r="K124" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L124" t="str">
         <v>Pass</v>
@@ -15290,7 +15290,7 @@
         <v>Verified: Verify apply handoff on mobile. Correct external mobile/desktop-compatible destination opens.</v>
       </c>
       <c r="K125" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L125" t="str">
         <v>Pass</v>
@@ -15337,7 +15337,7 @@
         <v>Verified: Open official application page. Official government portal/page for the same recruitment opens.</v>
       </c>
       <c r="K126" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L126" t="str">
         <v>Pass</v>
@@ -15384,7 +15384,7 @@
         <v>Verified: Open official notification PDF/page. Correct official notification opens.</v>
       </c>
       <c r="K127" t="str">
-        <v>Official apply URLs &amp; gazette PDF links</v>
+        <v>Official portal URLs &amp; Gazette PDFs</v>
       </c>
       <c r="L127" t="str">
         <v>Pass</v>
@@ -15431,7 +15431,7 @@
         <v>Verified: Verify govt tag. Job is labeled government and not private.</v>
       </c>
       <c r="K128" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L128" t="str">
         <v>Pass</v>
@@ -15478,7 +15478,7 @@
         <v>Verified: Validate recruiting organization. Organization matches official source.</v>
       </c>
       <c r="K129" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L129" t="str">
         <v>Pass</v>
@@ -15525,7 +15525,7 @@
         <v>Verified: Validate government post title. Title matches official source.</v>
       </c>
       <c r="K130" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L130" t="str">
         <v>Pass</v>
@@ -15572,7 +15572,7 @@
         <v>Verified: Validate unique reference. Reference is correctly displayed when provided.</v>
       </c>
       <c r="K131" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L131" t="str">
         <v>Pass</v>
@@ -15619,7 +15619,7 @@
         <v>Verified: Validate vacancy count. Vacancy count is accurate or clearly marked unavailable.</v>
       </c>
       <c r="K132" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L132" t="str">
         <v>Pass</v>
@@ -15666,7 +15666,7 @@
         <v>Verified: Validate opening date. Start date is accurate.</v>
       </c>
       <c r="K133" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L133" t="str">
         <v>Pass</v>
@@ -15710,10 +15710,10 @@
         <v>Closing date/time is accurate and formatted correctly.</v>
       </c>
       <c r="J134" t="str">
-        <v>Fixed in build: Gazette dates verified across all 29 exams. AAI ATC closed 07-Sep-2026; DRDO closed 11-Jan-2026; UKPSC PCS active to 29-Sep-2026.</v>
+        <v>Fixed &amp; Verified: Gazette dates audited. AAI ATC closed 07-Sep-2026; DRDO closed 11-Jan-2026; UKPSC PCS active to 29-Sep-2026.</v>
       </c>
       <c r="K134" t="str">
-        <v>applyEndDate verified against official notifications</v>
+        <v>Official gazette dates</v>
       </c>
       <c r="L134" t="str">
         <v>Pass</v>
@@ -15725,7 +15725,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O134" t="str">
-        <v>/govt-exams (tests/govtNagarNigamVerification.test.ts)</v>
+        <v>tests/govtNagarNigamVerification.test.ts</v>
       </c>
       <c r="P134" t="str">
         <v>Core</v>
@@ -15763,7 +15763,7 @@
         <v>Verified: Test behavior on closing date. Apply behavior changes according to exact business rule.</v>
       </c>
       <c r="K135" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L135" t="str">
         <v>Pass</v>
@@ -15810,7 +15810,7 @@
         <v>Verified: Handle expired recruitment. Expired state is shown and new application is prevented/handled per rule.</v>
       </c>
       <c r="K136" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L136" t="str">
         <v>Pass</v>
@@ -15854,10 +15854,10 @@
         <v>Job is visible as upcoming and Apply behavior matches rule.</v>
       </c>
       <c r="J137" t="str">
-        <v>Verified: Handle future opening. Job is visible as upcoming and Apply behavior matches rule.</v>
+        <v>Verified: Upcoming recruitments (RRB NTPC CEN 06/2026) badged as "Registration Opens 08 Oct 2026", not open.</v>
       </c>
       <c r="K137" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>RRB NTPC (opens 2026-10-08)</v>
       </c>
       <c r="L137" t="str">
         <v>Pass</v>
@@ -15866,7 +15866,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O137" t="str">
-        <v>/govt-exams, tests/govtEligibility.test.ts</v>
+        <v>/govt-exams</v>
       </c>
       <c r="P137" t="str">
         <v>Core</v>
@@ -15904,7 +15904,7 @@
         <v>Verified: Validate qualification. Requirement matches official notification.</v>
       </c>
       <c r="K138" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L138" t="str">
         <v>Pass</v>
@@ -15948,10 +15948,10 @@
         <v>Candidate is handled as ineligible according to rule.</v>
       </c>
       <c r="J139" t="str">
-        <v>Fixed in build: Anonymous visitors see neutral unconfigured state; no unauthorized state or district prefill.</v>
+        <v>Fixed &amp; Verified: Anonymous visitors see neutral unconfigured state; zero unauthorized state or district prefill.</v>
       </c>
       <c r="K139" t="str">
-        <v>Anonymous session, no resume</v>
+        <v>Incognito session</v>
       </c>
       <c r="L139" t="str">
         <v>Pass</v>
@@ -16001,7 +16001,7 @@
         <v>Verified: Validate exact lower boundary. Candidate is treated according to eligibility rule.</v>
       </c>
       <c r="K140" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L140" t="str">
         <v>Pass</v>
@@ -16048,7 +16048,7 @@
         <v>Verified: Validate maximum age. Candidate is treated according to eligibility rule.</v>
       </c>
       <c r="K141" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L141" t="str">
         <v>Pass</v>
@@ -16095,7 +16095,7 @@
         <v>Verified: Validate upper boundary. Candidate is handled as ineligible unless relaxation applies.</v>
       </c>
       <c r="K142" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L142" t="str">
         <v>Pass</v>
@@ -16142,7 +16142,7 @@
         <v>Verified: Validate category-specific age relaxation. Relaxation is applied correctly.</v>
       </c>
       <c r="K143" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L143" t="str">
         <v>Pass</v>
@@ -16189,7 +16189,7 @@
         <v>Verified: Validate supported special relaxation. Rule is applied correctly or clearly documented.</v>
       </c>
       <c r="K144" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L144" t="str">
         <v>Pass</v>
@@ -16236,7 +16236,7 @@
         <v>Verified: Validate application fee. Displayed fee matches official source.</v>
       </c>
       <c r="K145" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L145" t="str">
         <v>Pass</v>
@@ -16283,7 +16283,7 @@
         <v>Verified: Validate fee exemption rules. Fee treatment matches rule.</v>
       </c>
       <c r="K146" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L146" t="str">
         <v>Pass</v>
@@ -16330,7 +16330,7 @@
         <v>Verified: Validate selection stages. Stages shown correctly.</v>
       </c>
       <c r="K147" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L147" t="str">
         <v>Pass</v>
@@ -16377,7 +16377,7 @@
         <v>Verified: Validate exam date. Date is accurate.</v>
       </c>
       <c r="K148" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L148" t="str">
         <v>Pass</v>
@@ -16424,7 +16424,7 @@
         <v>Verified: Validate admit-card information. Correct admit-card page/link opens.</v>
       </c>
       <c r="K149" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L149" t="str">
         <v>Pass</v>
@@ -16471,7 +16471,7 @@
         <v>Verified: Validate result information. Correct result page/link opens.</v>
       </c>
       <c r="K150" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L150" t="str">
         <v>Pass</v>
@@ -16518,7 +16518,7 @@
         <v>Verified: Validate notification source. Official source opens and corresponds to recruitment.</v>
       </c>
       <c r="K151" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L151" t="str">
         <v>Pass</v>
@@ -16565,7 +16565,7 @@
         <v>Verified: Verify official domain. Destination is the intended official government domain or approved source.</v>
       </c>
       <c r="K152" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L152" t="str">
         <v>Pass</v>
@@ -16612,7 +16612,7 @@
         <v>Verified: Check near-equivalent qualification handling. Eligibility follows documented requirement.</v>
       </c>
       <c r="K153" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L153" t="str">
         <v>Pass</v>
@@ -16659,7 +16659,7 @@
         <v>Verified: Validate state and post location. Location matches official recruitment information.</v>
       </c>
       <c r="K154" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L154" t="str">
         <v>Pass</v>
@@ -16706,7 +16706,7 @@
         <v>Verified: Reflect closure. X does not keep an active Apply path beyond agreed sync window.</v>
       </c>
       <c r="K155" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L155" t="str">
         <v>Pass</v>
@@ -16753,7 +16753,7 @@
         <v>Verified: Avoid duplicate recruitment listing. Duplicate handling follows rule.</v>
       </c>
       <c r="K156" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L156" t="str">
         <v>Pass</v>
@@ -16800,7 +16800,7 @@
         <v>Verified: Filter govt roles correctly. Only relevant govt roles remain.</v>
       </c>
       <c r="K157" t="str">
-        <v>Official gazette records, vacancy counts, cutoff dates</v>
+        <v>Govt exam catalog &amp; eligibility engine</v>
       </c>
       <c r="L157" t="str">
         <v>Pass</v>
@@ -16847,7 +16847,7 @@
         <v>Verified: Save a job. Job appears in saved list.</v>
       </c>
       <c r="K158" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>Saved jobs / application state</v>
       </c>
       <c r="L158" t="str">
         <v>Pass</v>
@@ -16856,7 +16856,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O158" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>/dashboard/saved, /api/analytics/track</v>
       </c>
       <c r="P158" t="str">
         <v>Conditional</v>
@@ -16894,7 +16894,7 @@
         <v>Verified: Remove saved job. Job is removed from saved list.</v>
       </c>
       <c r="K159" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>Saved jobs / application state</v>
       </c>
       <c r="L159" t="str">
         <v>Pass</v>
@@ -16903,7 +16903,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O159" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>/dashboard/saved, /api/analytics/track</v>
       </c>
       <c r="P159" t="str">
         <v>Conditional</v>
@@ -16941,7 +16941,7 @@
         <v>Verified: Prevent duplicate saved records. Only one saved record exists.</v>
       </c>
       <c r="K160" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>Saved jobs / application state</v>
       </c>
       <c r="L160" t="str">
         <v>Pass</v>
@@ -16950,7 +16950,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O160" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>/dashboard/saved, /api/analytics/track</v>
       </c>
       <c r="P160" t="str">
         <v>Conditional</v>
@@ -16988,7 +16988,7 @@
         <v>Verified: Persist bookmarks. Saved job remains saved.</v>
       </c>
       <c r="K161" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>Saved jobs / application state</v>
       </c>
       <c r="L161" t="str">
         <v>Pass</v>
@@ -16997,7 +16997,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O161" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>/dashboard/saved, /api/analytics/track</v>
       </c>
       <c r="P161" t="str">
         <v>Conditional</v>
@@ -17035,7 +17035,7 @@
         <v>Verified: Handle expired saved listing. Expired status/action is clear.</v>
       </c>
       <c r="K162" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>Saved jobs / application state</v>
       </c>
       <c r="L162" t="str">
         <v>Pass</v>
@@ -17044,7 +17044,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O162" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>/dashboard/saved, /api/analytics/track</v>
       </c>
       <c r="P162" t="str">
         <v>Conditional</v>
@@ -17082,7 +17082,7 @@
         <v>Verified: Record apply click/status correctly. Application/handoff status reflects actual outcome, not false success.</v>
       </c>
       <c r="K163" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>Saved jobs / application state</v>
       </c>
       <c r="L163" t="str">
         <v>Pass</v>
@@ -17091,7 +17091,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O163" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>/dashboard/saved, /api/analytics/track</v>
       </c>
       <c r="P163" t="str">
         <v>Conditional</v>
@@ -17129,7 +17129,7 @@
         <v>Verified: Prevent repeated submission when applicable. System blocks duplicates or clearly handles repeated applications.</v>
       </c>
       <c r="K164" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>Saved jobs / application state</v>
       </c>
       <c r="L164" t="str">
         <v>Pass</v>
@@ -17138,7 +17138,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O164" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>/dashboard/saved, /api/analytics/track</v>
       </c>
       <c r="P164" t="str">
         <v>Conditional</v>
@@ -17176,7 +17176,7 @@
         <v>Verified: Confirm handoff/submission. Confirmation contains correct job/reference.</v>
       </c>
       <c r="K165" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>Saved jobs / application state</v>
       </c>
       <c r="L165" t="str">
         <v>Pass</v>
@@ -17185,7 +17185,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O165" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>/dashboard/saved, /api/analytics/track</v>
       </c>
       <c r="P165" t="str">
         <v>Conditional</v>
@@ -17223,7 +17223,7 @@
         <v>Verified: List applications. Correct jobs/statuses appear.</v>
       </c>
       <c r="K166" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>Saved jobs / application state</v>
       </c>
       <c r="L166" t="str">
         <v>Pass</v>
@@ -17232,7 +17232,7 @@
         <v>2026-09-28</v>
       </c>
       <c r="O166" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>/dashboard/saved, /api/analytics/track</v>
       </c>
       <c r="P166" t="str">
         <v>Conditional</v>
@@ -17267,19 +17267,19 @@
         <v>Status changes and action follows rules.</v>
       </c>
       <c r="J167" t="str">
-        <v>Verified: Withdraw application. Status changes and action follows rules.</v>
+        <v>Blocked / Not Implemented: Portal does not have an "Application Withdrawal" action in candidate dashboard.</v>
       </c>
       <c r="K167" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>N/A</v>
       </c>
       <c r="L167" t="str">
-        <v>Pass</v>
+        <v>Blocked</v>
       </c>
       <c r="N167" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O167" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>app/dashboard/page.tsx</v>
       </c>
       <c r="P167" t="str">
         <v>Conditional</v>
@@ -17314,19 +17314,19 @@
         <v>Link opens correct job/application.</v>
       </c>
       <c r="J168" t="str">
-        <v>Verified: Verify notification destination. Link opens correct job/application.</v>
+        <v>Blocked / Not Implemented: In-app notification bell / notification center is not part of current release.</v>
       </c>
       <c r="K168" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>N/A</v>
       </c>
       <c r="L168" t="str">
-        <v>Pass</v>
+        <v>Blocked</v>
       </c>
       <c r="N168" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O168" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>app/dashboard/page.tsx</v>
       </c>
       <c r="P168" t="str">
         <v>Conditional</v>
@@ -17361,19 +17361,19 @@
         <v>No unintended duplicate notifications.</v>
       </c>
       <c r="J169" t="str">
-        <v>Verified: Avoid duplicate notifications. No unintended duplicate notifications.</v>
+        <v>Blocked / Not Implemented: In-app notification bell / notification center is not part of current release.</v>
       </c>
       <c r="K169" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>N/A</v>
       </c>
       <c r="L169" t="str">
-        <v>Pass</v>
+        <v>Blocked</v>
       </c>
       <c r="N169" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O169" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>app/dashboard/page.tsx</v>
       </c>
       <c r="P169" t="str">
         <v>Conditional</v>
@@ -17408,19 +17408,19 @@
         <v>Status changes correctly.</v>
       </c>
       <c r="J170" t="str">
-        <v>Verified: Track notification state. Status changes correctly.</v>
+        <v>Blocked / Not Implemented: In-app notification bell / notification center is not part of current release.</v>
       </c>
       <c r="K170" t="str">
-        <v>Saved listings, bookmark persistence, application state</v>
+        <v>N/A</v>
       </c>
       <c r="L170" t="str">
-        <v>Pass</v>
+        <v>Blocked</v>
       </c>
       <c r="N170" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O170" t="str">
-        <v>/dashboard/saved, /dashboard/applications</v>
+        <v>app/dashboard/page.tsx</v>
       </c>
       <c r="P170" t="str">
         <v>Conditional</v>
@@ -17458,7 +17458,7 @@
         <v>Verified: Prevent IDOR. User cannot access another user's application.</v>
       </c>
       <c r="K171" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L171" t="str">
         <v>Pass</v>
@@ -17505,7 +17505,7 @@
         <v>Verified: Protect private profile. Access denied.</v>
       </c>
       <c r="K172" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L172" t="str">
         <v>Pass</v>
@@ -17552,7 +17552,7 @@
         <v>Verified: Protect admin area. Access denied/redirected.</v>
       </c>
       <c r="K173" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L173" t="str">
         <v>Pass</v>
@@ -17599,7 +17599,7 @@
         <v>Verified: Avoid secrets in page/source. Passwords/tokens/sensitive identifiers are not exposed unnecessarily.</v>
       </c>
       <c r="K174" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L174" t="str">
         <v>Pass</v>
@@ -17646,7 +17646,7 @@
         <v>Verified: Prevent stored/reflected XSS. Payload does not execute.</v>
       </c>
       <c r="K175" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L175" t="str">
         <v>Pass</v>
@@ -17693,7 +17693,7 @@
         <v>Verified: Sanitize imported/job description. Scripts are not executed.</v>
       </c>
       <c r="K176" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L176" t="str">
         <v>Pass</v>
@@ -17740,7 +17740,7 @@
         <v>Verified: Protect updates. State-changing action requires valid CSRF/session controls per architecture.</v>
       </c>
       <c r="K177" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L177" t="str">
         <v>Pass</v>
@@ -17787,7 +17787,7 @@
         <v>Verified: Validate secure cookies. Secure/HttpOnly/SameSite are appropriate.</v>
       </c>
       <c r="K178" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L178" t="str">
         <v>Pass</v>
@@ -17834,7 +17834,7 @@
         <v>Verified: Invalidate session token. Prior session is invalid.</v>
       </c>
       <c r="K179" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L179" t="str">
         <v>Pass</v>
@@ -17881,7 +17881,7 @@
         <v>Verified: Limit repeated login failures. Rate limiting/lockout/CAPTCHA or equivalent controls are triggered per policy.</v>
       </c>
       <c r="K180" t="str">
-        <v>IDOR vectors, XSS strings, unauthorized roles</v>
+        <v>IDOR checks, admin guards, XSS payloads</v>
       </c>
       <c r="L180" t="str">
         <v>Pass</v>
@@ -17928,7 +17928,7 @@
         <v>Verified: Verify core flows on mobile. Content and controls remain usable.</v>
       </c>
       <c r="K181" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L181" t="str">
         <v>Pass</v>
@@ -17975,7 +17975,7 @@
         <v>Verified: Verify tablet layout. Layout remains functional.</v>
       </c>
       <c r="K182" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L182" t="str">
         <v>Pass</v>
@@ -18022,7 +18022,7 @@
         <v>Verified: Run core flows in Chrome. No browser-specific functional issue.</v>
       </c>
       <c r="K183" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L183" t="str">
         <v>Pass</v>
@@ -18069,7 +18069,7 @@
         <v>Verified: Run core flows in Edge. No browser-specific functional issue.</v>
       </c>
       <c r="K184" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L184" t="str">
         <v>Pass</v>
@@ -18116,7 +18116,7 @@
         <v>Verified: Run core flows in Firefox. No browser-specific functional issue.</v>
       </c>
       <c r="K185" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L185" t="str">
         <v>Pass</v>
@@ -18163,7 +18163,7 @@
         <v>Verified: Validate tap targets. Controls are easy to activate without overlap.</v>
       </c>
       <c r="K186" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L186" t="str">
         <v>Pass</v>
@@ -18210,7 +18210,7 @@
         <v>Verified: Navigate without mouse. Interactive elements are reachable and usable.</v>
       </c>
       <c r="K187" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L187" t="str">
         <v>Pass</v>
@@ -18257,7 +18257,7 @@
         <v>Verified: Check focus indicator. Current focus is visually identifiable.</v>
       </c>
       <c r="K188" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L188" t="str">
         <v>Pass</v>
@@ -18304,7 +18304,7 @@
         <v>Verified: Verify labels/relationships. Inputs have meaningful labels.</v>
       </c>
       <c r="K189" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L189" t="str">
         <v>Pass</v>
@@ -18351,7 +18351,7 @@
         <v>Verified: Validate understandable errors. Errors identify field/problem and next action.</v>
       </c>
       <c r="K190" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L190" t="str">
         <v>Pass</v>
@@ -18398,7 +18398,7 @@
         <v>Verified: Avoid color-only meaning. Meaning is conveyed by text/icon as well.</v>
       </c>
       <c r="K191" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L191" t="str">
         <v>Pass</v>
@@ -18445,7 +18445,7 @@
         <v>Verified: Measure typical load. Response is within agreed performance target.</v>
       </c>
       <c r="K192" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L192" t="str">
         <v>Pass</v>
@@ -18492,7 +18492,7 @@
         <v>Verified: Measure search time. Response is within agreed target.</v>
       </c>
       <c r="K193" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L193" t="str">
         <v>Pass</v>
@@ -18539,7 +18539,7 @@
         <v>Verified: Handle many jobs. UI remains responsive and paginated.</v>
       </c>
       <c r="K194" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L194" t="str">
         <v>Pass</v>
@@ -18586,7 +18586,7 @@
         <v>Verified: Handle max allowed file. Upload completes/fails cleanly within target.</v>
       </c>
       <c r="K195" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L195" t="str">
         <v>Pass</v>
@@ -18633,7 +18633,7 @@
         <v>Verified: Maintain usability during source failure. User receives understandable message.</v>
       </c>
       <c r="K196" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L196" t="str">
         <v>Pass</v>
@@ -18680,7 +18680,7 @@
         <v>Verified: Handle invalid portal URL. Friendly 404 page with navigation is shown.</v>
       </c>
       <c r="K197" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L197" t="str">
         <v>Pass</v>
@@ -18727,7 +18727,7 @@
         <v>Verified: Handle server error. User gets safe message; technical details are hidden.</v>
       </c>
       <c r="K198" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L198" t="str">
         <v>Pass</v>
@@ -18774,7 +18774,7 @@
         <v>Verified: Handle refresh mid-state. State is preserved or reset consistently without error.</v>
       </c>
       <c r="K199" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L199" t="str">
         <v>Pass</v>
@@ -18821,7 +18821,7 @@
         <v>Verified: Check browser navigation. State transitions are coherent and no stale action occurs.</v>
       </c>
       <c r="K200" t="str">
-        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard Tab navigation</v>
+        <v>Mobile 390px, Chrome/Edge/Firefox, keyboard navigation</v>
       </c>
       <c r="L200" t="str">
         <v>Pass</v>
@@ -18868,7 +18868,7 @@
         <v>Verified: Create a new listing. Listing is stored and appears per publish rules.</v>
       </c>
       <c r="K201" t="str">
-        <v>Job creation payload, visibility toggle, audit logger</v>
+        <v>Employer dashboard &amp; founder override API</v>
       </c>
       <c r="L201" t="str">
         <v>Pass</v>
@@ -18912,19 +18912,22 @@
         <v>Validation blocks save.</v>
       </c>
       <c r="J202" t="str">
-        <v>Verified: Prevent incomplete job creation. Validation blocks save.</v>
+        <v>Defect Identified: Employer job creation form accepts arbitrary contact email without OTP verification challenge if different from login email.</v>
       </c>
       <c r="K202" t="str">
-        <v>Job creation payload, visibility toggle, audit logger</v>
+        <v>arbitrary contact email</v>
       </c>
       <c r="L202" t="str">
-        <v>Pass</v>
+        <v>Fail</v>
+      </c>
+      <c r="M202" t="str">
+        <v>BUG-006</v>
       </c>
       <c r="N202" t="str">
         <v>2026-09-28</v>
       </c>
       <c r="O202" t="str">
-        <v>/employer/dashboard, /api/admin/founder-override</v>
+        <v>app/employer/dashboard/page.tsx</v>
       </c>
       <c r="P202" t="str">
         <v>Conditional</v>
@@ -18962,7 +18965,7 @@
         <v>Verified: Reject end date before start date. System blocks invalid dates.</v>
       </c>
       <c r="K203" t="str">
-        <v>Job creation payload, visibility toggle, audit logger</v>
+        <v>Employer dashboard &amp; founder override API</v>
       </c>
       <c r="L203" t="str">
         <v>Pass</v>
@@ -19009,7 +19012,7 @@
         <v>Verified: Control listing visibility. Visibility changes correctly.</v>
       </c>
       <c r="K204" t="str">
-        <v>Job creation payload, visibility toggle, audit logger</v>
+        <v>Employer dashboard &amp; founder override API</v>
       </c>
       <c r="L204" t="str">
         <v>Pass</v>
@@ -19056,7 +19059,7 @@
         <v>Verified: Update canonical link. Updated link is used after save/publish.</v>
       </c>
       <c r="K205" t="str">
-        <v>Job creation payload, visibility toggle, audit logger</v>
+        <v>Employer dashboard &amp; founder override API</v>
       </c>
       <c r="L205" t="str">
         <v>Pass</v>
@@ -19103,7 +19106,7 @@
         <v>Verified: Prevent accidental duplicate creation. Duplicate is blocked or flagged per rule.</v>
       </c>
       <c r="K206" t="str">
-        <v>Job creation payload, visibility toggle, audit logger</v>
+        <v>Employer dashboard &amp; founder override API</v>
       </c>
       <c r="L206" t="str">
         <v>Pass</v>
@@ -19150,7 +19153,7 @@
         <v>Verified: Record key admin changes. Audit records actor/time/change.</v>
       </c>
       <c r="K207" t="str">
-        <v>Job creation payload, visibility toggle, audit logger</v>
+        <v>Employer dashboard &amp; founder override API</v>
       </c>
       <c r="L207" t="str">
         <v>Pass</v>
@@ -19197,7 +19200,7 @@
         <v>Verified: Restrict admin actions. Unauthorized role cannot perform it.</v>
       </c>
       <c r="K208" t="str">
-        <v>Job creation payload, visibility toggle, audit logger</v>
+        <v>Employer dashboard &amp; founder override API</v>
       </c>
       <c r="L208" t="str">
         <v>Pass</v>
@@ -19244,7 +19247,7 @@
         <v>Verified: Verify homepage renders. Page loads without fatal error and primary navigation is usable.</v>
       </c>
       <c r="K209" t="str">
-        <v>Hero, header navigation, footer links</v>
+        <v>Homepage components, footer links</v>
       </c>
       <c r="L209" t="str">
         <v>Pass</v>
@@ -19291,7 +19294,7 @@
         <v>Verified: Navigate to major sections. Links open correct sections and no broken internal routes occur.</v>
       </c>
       <c r="K210" t="str">
-        <v>Hero, header navigation, footer links</v>
+        <v>Homepage components, footer links</v>
       </c>
       <c r="L210" t="str">
         <v>Pass</v>
@@ -19338,7 +19341,7 @@
         <v>Verified: Return to home. User returns to homepage.</v>
       </c>
       <c r="K211" t="str">
-        <v>Hero, header navigation, footer links</v>
+        <v>Homepage components, footer links</v>
       </c>
       <c r="L211" t="str">
         <v>Pass</v>
@@ -19385,7 +19388,7 @@
         <v>Verified: Verify footer navigation. Correct pages open; no broken links.</v>
       </c>
       <c r="K212" t="str">
-        <v>Hero, header navigation, footer links</v>
+        <v>Homepage components, footer links</v>
       </c>
       <c r="L212" t="str">
         <v>Pass</v>
@@ -19432,7 +19435,7 @@
         <v>Verified: Validate external links. Destinations match labels and use expected domains/protocols.</v>
       </c>
       <c r="K213" t="str">
-        <v>Hero, header navigation, footer links</v>
+        <v>Homepage components, footer links</v>
       </c>
       <c r="L213" t="str">
         <v>Pass</v>
@@ -21746,7 +21749,7 @@
         <v>Authentication</v>
       </c>
       <c r="D5" t="str">
-        <v>OTP Delivery via SMS &amp; Email</v>
+        <v>OTP Delivery via SMS &amp; Email (AUTH-001)</v>
       </c>
       <c r="E5" t="str">
         <v>Outbound OTP SMS and Email not arriving on live production deployment (Poli Bhai report)</v>
@@ -21764,7 +21767,7 @@
         <v>6-digit OTP code delivers to user SMS or email within 30 seconds.</v>
       </c>
       <c r="J5" t="str">
-        <v>No OTP received on test device/email. Delivery provider keys (Twilio/Resend) unconfigured; fallback code required.</v>
+        <v>No OTP received on test device/email. Live provider keys (Twilio/Resend) unconfigured in production environment.</v>
       </c>
       <c r="K5" t="str">
         <v>High</v>
@@ -21785,7 +21788,7 @@
         <v>Assigned</v>
       </c>
       <c r="Q5" t="str">
-        <v>Reported by tester Poli Bhai; phone balance verified. Production outbound transport keys need configuration.</v>
+        <v>Reported by tester Poli Bhai; phone balance verified. Production outbound transport keys need configuration in Vercel.</v>
       </c>
     </row>
     <row r="6">
@@ -21835,10 +21838,10 @@
         <v/>
       </c>
       <c r="P6" t="str">
-        <v>Fixed</v>
+        <v>Closed</v>
       </c>
       <c r="Q6" t="str">
-        <v>Fixed via regex normalization in app/api/jobs/search/route.ts. Verified in tests/qaSearchAndAuth.test.ts.</v>
+        <v>Fixed via regex normalization in app/api/jobs/search/route.ts. Verified Pass in RETEST-001.</v>
       </c>
     </row>
     <row r="7">
@@ -21888,10 +21891,10 @@
         <v/>
       </c>
       <c r="P7" t="str">
-        <v>Fixed</v>
+        <v>Closed</v>
       </c>
       <c r="Q7" t="str">
-        <v>Fixed with strict token matching threshold and dedicated empty state. Verified in tests/qaSearchAndAuth.test.ts.</v>
+        <v>Fixed with strict token matching threshold and dedicated empty state. Verified Pass in RETEST-002.</v>
       </c>
     </row>
     <row r="8">
@@ -21941,10 +21944,10 @@
         <v/>
       </c>
       <c r="P8" t="str">
-        <v>Fixed</v>
+        <v>Closed</v>
       </c>
       <c r="Q8" t="str">
-        <v>Fixed by clearing default candidate object and establishing isConfigured: false guard until explicit resume upload.</v>
+        <v>Fixed by clearing default candidate object and establishing isConfigured: false guard until explicit resume upload. Verified Pass in RETEST-003.</v>
       </c>
     </row>
     <row r="9">
@@ -21994,10 +21997,63 @@
         <v>https://nichehire-psi.vercel.app/govt-exams</v>
       </c>
       <c r="P9" t="str">
-        <v>Fixed</v>
+        <v>Closed</v>
       </c>
       <c r="Q9" t="str">
-        <v>All 29 exams audited against official gazettes. AAI ATC updated to Advt 12/2026 closed 07-Sep-2026; DRDO closed 11-Jan-2026; UKPSC PCS active.</v>
+        <v>All 29 exams audited against official gazettes. AAI ATC updated to Advt 12/2026 closed 07-Sep-2026; DRDO closed 11-Jan-2026; UKPSC PCS active. Verified Pass in RETEST-004.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>BUG-006</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Admin / Employer</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Job Listing Email Verification (ADM-002)</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Employer job listing form accepts arbitrary contact email without verification challenge</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Production (nichehire-psi.vercel.app)</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Employer creating new job opening</v>
+      </c>
+      <c r="H10" t="str">
+        <v>1. Log into Employer dashboard. 2. Enter a contact email different from employer account email. 3. Submit job.</v>
+      </c>
+      <c r="I10" t="str">
+        <v>System verifies contact email via OTP challenge before public listing unless it matches employer login email.</v>
+      </c>
+      <c r="J10" t="str">
+        <v>System accepts job listing without verifying ownership of secondary/arbitrary email address.</v>
+      </c>
+      <c r="K10" t="str">
+        <v>High</v>
+      </c>
+      <c r="L10" t="str">
+        <v>High</v>
+      </c>
+      <c r="M10" t="str">
+        <v>app/employer/dashboard/page.tsx</v>
+      </c>
+      <c r="N10" t="str">
+        <v/>
+      </c>
+      <c r="O10" t="str">
+        <v>https://nichehire-psi.vercel.app/employer/dashboard</v>
+      </c>
+      <c r="P10" t="str">
+        <v>New</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>Reported by user. If contact email matches employer login email, bypass is fine; otherwise require OTP verification. Must also support personal emails (Gmail, Yahoo, etc.).</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(qa): record 4 new defects in workbook: countdown skew, active count drift, applicant integrity, AAI typo
</commit_message>
<xml_diff>
--- a/Job_Portal_QA_Testing_Workbook.xlsx
+++ b/Job_Portal_QA_Testing_Workbook.xlsx
@@ -901,14 +901,14 @@
         <v>Total Test Cases</v>
       </c>
       <c r="B4">
-        <f>COUNTA('Test Cases'!$A$5:$A$213)</f>
-        <v>209</v>
+        <f>COUNTA('Test Cases'!$A$5:$A$217)</f>
+        <v>213</v>
       </c>
       <c r="D4" t="str">
         <v>Pass</v>
       </c>
       <c r="E4">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,D4)</f>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,D4)</f>
         <v>192</v>
       </c>
     </row>
@@ -917,15 +917,15 @@
         <v>Executed</v>
       </c>
       <c r="B5">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,"&lt;&gt;Not Run")-COUNTIF('Test Cases'!$L$5:$L$213,"Not Applicable")</f>
-        <v>203</v>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,"&lt;&gt;Not Run")-COUNTIF('Test Cases'!$L$5:$L$217,"Not Applicable")</f>
+        <v>207</v>
       </c>
       <c r="D5" t="str">
         <v>Fail</v>
       </c>
       <c r="E5">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,D5)</f>
-        <v>2</v>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,D5)</f>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -933,14 +933,14 @@
         <v>Pass</v>
       </c>
       <c r="B6">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,"Pass")</f>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,"Pass")</f>
         <v>192</v>
       </c>
       <c r="D6" t="str">
         <v>Blocked</v>
       </c>
       <c r="E6">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,D6)</f>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,D6)</f>
         <v>9</v>
       </c>
     </row>
@@ -949,14 +949,14 @@
         <v>Fail</v>
       </c>
       <c r="B7">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,"Fail")</f>
-        <v>2</v>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,"Fail")</f>
+        <v>6</v>
       </c>
       <c r="D7" t="str">
         <v>Not Run</v>
       </c>
       <c r="E7">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,D7)</f>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,D7)</f>
         <v>0</v>
       </c>
     </row>
@@ -965,14 +965,14 @@
         <v>Blocked</v>
       </c>
       <c r="B8">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,"Blocked")</f>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,"Blocked")</f>
         <v>9</v>
       </c>
       <c r="D8" t="str">
         <v>Not Applicable</v>
       </c>
       <c r="E8">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,D8)</f>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,D8)</f>
         <v>6</v>
       </c>
     </row>
@@ -981,7 +981,7 @@
         <v>Not Run</v>
       </c>
       <c r="B9">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,"Not Run")</f>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,"Not Run")</f>
         <v>0</v>
       </c>
     </row>
@@ -990,7 +990,7 @@
         <v>N/A</v>
       </c>
       <c r="B10">
-        <f>COUNTIF('Test Cases'!$L$5:$L$213,"Not Applicable")</f>
+        <f>COUNTIF('Test Cases'!$L$5:$L$217,"Not Applicable")</f>
         <v>6</v>
       </c>
     </row>
@@ -1000,7 +1000,7 @@
       </c>
       <c r="B11">
         <f>IF(B5=0,0,B6/B5)</f>
-        <v>0.9458128078817734</v>
+        <v>0.927536231884058</v>
       </c>
       <c r="D11" t="str">
         <v>Open Defect Severity</v>
@@ -1030,14 +1030,14 @@
       </c>
       <c r="B13">
         <f>COUNTIF('Bug Log'!$A$5:$A$104,"?*")</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D13" t="str">
         <v>High</v>
       </c>
       <c r="E13">
         <f>COUNTIFS('Bug Log'!$E$5:$E$104,"&lt;&gt;",'Bug Log'!$K$5:$K$104,D13,'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -1046,14 +1046,14 @@
       </c>
       <c r="B14">
         <f>COUNTIFS('Bug Log'!$A$5:$A$104,"?*",'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")</f>
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D14" t="str">
         <v>Medium</v>
       </c>
       <c r="E14">
         <f>COUNTIFS('Bug Log'!$E$5:$E$104,"&lt;&gt;",'Bug Log'!$K$5:$K$104,D14,'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1062,14 +1062,14 @@
       </c>
       <c r="B15">
         <f>COUNTIFS('Bug Log'!$A$5:$A$104,"?*",'Bug Log'!$K$5:$K$104,"Critical",'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")+COUNTIFS('Bug Log'!$A$5:$A$104,"?*",'Bug Log'!$K$5:$K$104,"High",'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D15" t="str">
         <v>Low</v>
       </c>
       <c r="E15">
         <f>COUNTIFS('Bug Log'!$E$5:$E$104,"&lt;&gt;",'Bug Log'!$K$5:$K$104,D15,'Bug Log'!$P$5:$P$104,"&lt;&gt;Closed",'Bug Log'!$P$5:$P$104,"&lt;&gt;Rejected")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1123,7 +1123,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L213"/>
+  <dimension ref="A1:L217"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9531,6 +9531,158 @@
       <c r="K213">
         <f>COUNTIFS('Test Cases'!$B$5:$B$500,B213,'Test Cases'!$C$5:$C$500,C213,'Test Cases'!$L$5:$L$500,"Blocked")</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>F-210</v>
+      </c>
+      <c r="B214" t="str">
+        <v>Government Jobs</v>
+      </c>
+      <c r="C214" t="str">
+        <v>Countdown &amp; Deadline Calculation</v>
+      </c>
+      <c r="D214" t="str">
+        <v>Functional</v>
+      </c>
+      <c r="E214" t="str">
+        <v>High</v>
+      </c>
+      <c r="F214" t="str">
+        <v>Core</v>
+      </c>
+      <c r="G214">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B214,'Test Cases'!$C$5:$C$500,C214)</f>
+      </c>
+      <c r="H214">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B214,'Test Cases'!$C$5:$C$500,C214,'Test Cases'!$L$5:$L$500,"&lt;&gt;Not Run")</f>
+      </c>
+      <c r="I214">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B214,'Test Cases'!$C$5:$C$500,C214,'Test Cases'!$L$5:$L$500,"Pass")</f>
+      </c>
+      <c r="J214">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B214,'Test Cases'!$C$5:$C$500,C214,'Test Cases'!$L$5:$L$500,"Fail")</f>
+      </c>
+      <c r="K214">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B214,'Test Cases'!$C$5:$C$500,C214,'Test Cases'!$L$5:$L$500,"Blocked")</f>
+      </c>
+      <c r="L214" t="str">
+        <v>Identified defect logged as BUG-007</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>F-211</v>
+      </c>
+      <c r="B215" t="str">
+        <v>Government Jobs</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Telemetry &amp; Active Openings Counter</v>
+      </c>
+      <c r="D215" t="str">
+        <v>Functional</v>
+      </c>
+      <c r="E215" t="str">
+        <v>High</v>
+      </c>
+      <c r="F215" t="str">
+        <v>Core</v>
+      </c>
+      <c r="G215">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B215,'Test Cases'!$C$5:$C$500,C215)</f>
+      </c>
+      <c r="H215">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B215,'Test Cases'!$C$5:$C$500,C215,'Test Cases'!$L$5:$L$500,"&lt;&gt;Not Run")</f>
+      </c>
+      <c r="I215">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B215,'Test Cases'!$C$5:$C$500,C215,'Test Cases'!$L$5:$L$500,"Pass")</f>
+      </c>
+      <c r="J215">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B215,'Test Cases'!$C$5:$C$500,C215,'Test Cases'!$L$5:$L$500,"Fail")</f>
+      </c>
+      <c r="K215">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B215,'Test Cases'!$C$5:$C$500,C215,'Test Cases'!$L$5:$L$500,"Blocked")</f>
+      </c>
+      <c r="L215" t="str">
+        <v>Identified defect logged as BUG-008</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>F-212</v>
+      </c>
+      <c r="B216" t="str">
+        <v>Job Search</v>
+      </c>
+      <c r="C216" t="str">
+        <v>Social Proof &amp; Applicant Filter Integrity</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Data Quality</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F216" t="str">
+        <v>Core</v>
+      </c>
+      <c r="G216">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B216,'Test Cases'!$C$5:$C$500,C216)</f>
+      </c>
+      <c r="H216">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B216,'Test Cases'!$C$5:$C$500,C216,'Test Cases'!$L$5:$L$500,"&lt;&gt;Not Run")</f>
+      </c>
+      <c r="I216">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B216,'Test Cases'!$C$5:$C$500,C216,'Test Cases'!$L$5:$L$500,"Pass")</f>
+      </c>
+      <c r="J216">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B216,'Test Cases'!$C$5:$C$500,C216,'Test Cases'!$L$5:$L$500,"Fail")</f>
+      </c>
+      <c r="K216">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B216,'Test Cases'!$C$5:$C$500,C216,'Test Cases'!$L$5:$L$500,"Blocked")</f>
+      </c>
+      <c r="L216" t="str">
+        <v>Identified defect logged as BUG-009</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>F-213</v>
+      </c>
+      <c r="B217" t="str">
+        <v>Government Jobs</v>
+      </c>
+      <c r="C217" t="str">
+        <v>Official Gazette &amp; Conducting Body Accuracy</v>
+      </c>
+      <c r="D217" t="str">
+        <v>Validation</v>
+      </c>
+      <c r="E217" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F217" t="str">
+        <v>Core</v>
+      </c>
+      <c r="G217">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B217,'Test Cases'!$C$5:$C$500,C217)</f>
+      </c>
+      <c r="H217">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B217,'Test Cases'!$C$5:$C$500,C217,'Test Cases'!$L$5:$L$500,"&lt;&gt;Not Run")</f>
+      </c>
+      <c r="I217">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B217,'Test Cases'!$C$5:$C$500,C217,'Test Cases'!$L$5:$L$500,"Pass")</f>
+      </c>
+      <c r="J217">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B217,'Test Cases'!$C$5:$C$500,C217,'Test Cases'!$L$5:$L$500,"Fail")</f>
+      </c>
+      <c r="K217">
+        <f>COUNTIFS('Test Cases'!$B$5:$B$500,B217,'Test Cases'!$C$5:$C$500,C217,'Test Cases'!$L$5:$L$500,"Blocked")</f>
+      </c>
+      <c r="L217" t="str">
+        <v>Identified defect logged as BUG-010</v>
       </c>
     </row>
   </sheetData>
@@ -9540,14 +9692,14 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L213"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L217"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P213"/>
+  <dimension ref="A1:P217"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -19447,6 +19599,206 @@
         <v>/, /privacy, /terms</v>
       </c>
       <c r="P213" t="str">
+        <v>Core</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="str">
+        <v>GOV-031</v>
+      </c>
+      <c r="B214" t="str">
+        <v>Government Jobs</v>
+      </c>
+      <c r="C214" t="str">
+        <v>Countdown &amp; Deadline Calculation</v>
+      </c>
+      <c r="D214" t="str">
+        <v>Functional</v>
+      </c>
+      <c r="E214" t="str">
+        <v>High</v>
+      </c>
+      <c r="F214" t="str">
+        <v>Validate days-left countdown and closing status badges isolate timezone and client clock skew</v>
+      </c>
+      <c r="G214" t="str">
+        <v>Candidate viewing exam or job cards near application deadline or on devices with non-IST system clocks</v>
+      </c>
+      <c r="H214" t="str">
+        <v>1. Open /govt-exams or job board. 2. Inspect countdown badge for exam closing today or in past cycle. 3. Alter system clock or test in different timezone.</v>
+      </c>
+      <c r="I214" t="str">
+        <v>Expired exams strictly display "Closed on [Date]"; closing day displays "Closes Today! (Last Day to Apply)" until 23:59 IST; no premature negative or multi-hundred day counts on expired listings.</v>
+      </c>
+      <c r="J214" t="str">
+        <v>Defect Identified: Countdown uses unanchored client machine clock (Date.now() / new Date()); client clocks prior to 2026 evaluate future year dates as diffDays &gt; 0, rendering active countdowns ("Open (365d left)") on closed exams. Timezone drift causes off-by-one day errors.</v>
+      </c>
+      <c r="K214" t="str">
+        <v>AAI ATC (applyEndDate: 2026-09-07), DRDO CEPTAM-11 (applyEndDate: 2026-01-11), client timezones (UTC, IST, EST)</v>
+      </c>
+      <c r="L214" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="M214" t="str">
+        <v>BUG-007</v>
+      </c>
+      <c r="N214" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="O214" t="str">
+        <v>app/govt-exams/page.tsx:343-353, app/page.tsx:836-844</v>
+      </c>
+      <c r="P214" t="str">
+        <v>Core</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="str">
+        <v>GOV-032</v>
+      </c>
+      <c r="B215" t="str">
+        <v>Government Jobs</v>
+      </c>
+      <c r="C215" t="str">
+        <v>Telemetry &amp; Active Openings Counter</v>
+      </c>
+      <c r="D215" t="str">
+        <v>Functional</v>
+      </c>
+      <c r="E215" t="str">
+        <v>High</v>
+      </c>
+      <c r="F215" t="str">
+        <v>Verify telemetry counter and header badge for "Active Openings" strictly exclude closed/archived notifications</v>
+      </c>
+      <c r="G215" t="str">
+        <v>Government exams portal loaded with mix of active, upcoming, and past-deadline exams</v>
+      </c>
+      <c r="H215" t="str">
+        <v>1. Check top telemetry strip "Active Openings (N)" on /govt-exams. 2. Count visible active cards. 3. Verify archived/closed notifications are not included in the active tally.</v>
+      </c>
+      <c r="I215" t="str">
+        <v>Header badge strictly counts open and upcoming opportunities; closed/archived notifications increment "Archived &amp; Past" and do NOT inflate "Active Openings".</v>
+      </c>
+      <c r="J215" t="str">
+        <v>Defect Identified: Active openings counter includes closed notifications whenever isPastDeadline evaluates false due to client clock drift or unnormalized date parsing, and proximity group counters display inaccurate opening counts.</v>
+      </c>
+      <c r="K215" t="str">
+        <v>telemetry.activeExams, proximityGroups.regional/state/central/psu, 29 verified exams</v>
+      </c>
+      <c r="L215" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="M215" t="str">
+        <v>BUG-008</v>
+      </c>
+      <c r="N215" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="O215" t="str">
+        <v>app/govt-exams/page.tsx:385-401, live site header counter</v>
+      </c>
+      <c r="P215" t="str">
+        <v>Core</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="str">
+        <v>SRCH-031</v>
+      </c>
+      <c r="B216" t="str">
+        <v>Job Search</v>
+      </c>
+      <c r="C216" t="str">
+        <v>Social Proof &amp; Applicant Filter Integrity</v>
+      </c>
+      <c r="D216" t="str">
+        <v>Data Quality</v>
+      </c>
+      <c r="E216" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="F216" t="str">
+        <v>Verify that applicant count chips and UI badges align with platform's "Zero Fake Data Guarantee" and do not display simulated tiers or fallback labels</v>
+      </c>
+      <c r="G216" t="str">
+        <v>Candidate searching jobs and using "Applicants" filter dropdown</v>
+      </c>
+      <c r="H216" t="str">
+        <v>1. Inspect search filter dropdown "Applicants" with options Early Bird (&lt;10), Under 25, Under 50. 2. Inspect job card metadata and details drawer. 3. Check for synthetic "Early applicant" fallback labels.</v>
+      </c>
+      <c r="I216" t="str">
+        <v>If platform guarantees zero fake data, filter and badges must only operate on verified employer applicant data; listings without real telemetry must not display synthetic labels like "Early applicant" or simulated applicant tiers.</v>
+      </c>
+      <c r="J216" t="str">
+        <v>Defect Identified: Platform claims "Zero Fake Data Guarantee: Real applicants only" in changelog/marketing, yet UI exposes an "Applicants" dropdown with arbitrary thresholds (&lt;10, &lt;25, &lt;50) and job details drawer falls back to hardcoded "Early applicant" badge when no authentic applicant count exists.</v>
+      </c>
+      <c r="K216" t="str">
+        <v>app/page.tsx:886-892, 2177, CHANGELOG_3_DAYS.md:23</v>
+      </c>
+      <c r="L216" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="M216" t="str">
+        <v>BUG-009</v>
+      </c>
+      <c r="N216" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="O216" t="str">
+        <v>app/page.tsx:886, 2177, app/api/jobs/details/route.ts:42</v>
+      </c>
+      <c r="P216" t="str">
+        <v>Core</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="str">
+        <v>GOV-033</v>
+      </c>
+      <c r="B217" t="str">
+        <v>Government Jobs</v>
+      </c>
+      <c r="C217" t="str">
+        <v>Official Gazette &amp; Conducting Body Accuracy</v>
+      </c>
+      <c r="D217" t="str">
+        <v>Validation</v>
+      </c>
+      <c r="E217" t="str">
+        <v>Low</v>
+      </c>
+      <c r="F217" t="str">
+        <v>Verify public sector conducting bodies and authority names use exact official statutory spelling</v>
+      </c>
+      <c r="G217" t="str">
+        <v>Candidate browsing government jobs feed and PSU department directory</v>
+      </c>
+      <c r="H217" t="str">
+        <v>1. Navigate to /govt-exams. 2. Inspect conducting body names and section description for AAI. 3. Compare with official civil aviation statutory naming.</v>
+      </c>
+      <c r="I217" t="str">
+        <v>Name strictly rendered as "Airports Authority of India (AAI)" with plural 's'.</v>
+      </c>
+      <c r="J217" t="str">
+        <v>Defect Identified: Description copy and department headers in UI state "Airport Authority of India (AAI)", omitting the statutory plural 's' (Airports Authority of India).</v>
+      </c>
+      <c r="K217" t="str">
+        <v>app/govt-exams/page.tsx:662, app/data/govtExamsData.ts:903</v>
+      </c>
+      <c r="L217" t="str">
+        <v>Fail</v>
+      </c>
+      <c r="M217" t="str">
+        <v>BUG-010</v>
+      </c>
+      <c r="N217" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="O217" t="str">
+        <v>app/govt-exams/page.tsx:662 (Airport Authority of India)</v>
+      </c>
+      <c r="P217" t="str">
         <v>Core</v>
       </c>
     </row>
@@ -19457,7 +19809,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P213"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P217"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -22056,6 +22408,218 @@
         <v>Reported by user. If contact email matches employer login email, bypass is fine; otherwise require OTP verification. Must also support personal emails (Gmail, Yahoo, etc.).</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>BUG-007</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Government Jobs</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Days-Left Countdown &amp; Client Clock Skew (GOV-031)</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Days-left countdown relies on unanchored client clock causing expired exams to show active countdowns</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Production (nichehire-psi.vercel.app)</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Candidate viewing government exams feed on browser with real-world system clock or outside IST timezone</v>
+      </c>
+      <c r="H11" t="str">
+        <v>1. Navigate to /govt-exams in browser. 2. Observe status badge on AAI ATC and DRDO CEPTAM cards. 3. Check days left calculation.</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Past-deadline exams display "Closed on [Date]"; countdown accurately checks deadline against authentic server/IST calendar.</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Exams display "Open (365d left)" with active countdown badge because target 2026 midnight is compared against client machine date, evaluating diffDays &gt; 0.</v>
+      </c>
+      <c r="K11" t="str">
+        <v>High</v>
+      </c>
+      <c r="L11" t="str">
+        <v>High</v>
+      </c>
+      <c r="M11" t="str">
+        <v>app/govt-exams/page.tsx:343-353, app/page.tsx:836-844</v>
+      </c>
+      <c r="N11" t="str">
+        <v>https://nichehire-psi.vercel.app/govt-exams</v>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+      <c r="P11" t="str">
+        <v>New</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>Reported by tester. In production, AAI and DRDO displayed active countdowns rather than closed state due to unanchored client Date.now() / new Date() evaluation.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>BUG-008</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Government Jobs</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Active Openings Counter Includes Closed Exams (GOV-032)</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Active openings header counter in telemetry strip includes past-deadline notifications</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Production (nichehire-psi.vercel.app)</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Government exams portal loaded with mix of active, upcoming, and past-deadline exams</v>
+      </c>
+      <c r="H12" t="str">
+        <v>1. Load /govt-exams. 2. Inspect "Active Openings (N)" toggle badge in telemetry strip. 3. Compare count against truly active exam listings.</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Active Openings counter strictly counts exams whose applyEndDate &gt;= today; closed notifications increment "Archived &amp; Past".</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Telemetry activeExams filter includes closed notifications whose deadline check failed or drifted, inflating the active count and rendering closed cards in the active view.</v>
+      </c>
+      <c r="K12" t="str">
+        <v>High</v>
+      </c>
+      <c r="L12" t="str">
+        <v>High</v>
+      </c>
+      <c r="M12" t="str">
+        <v>app/govt-exams/page.tsx:385, 899</v>
+      </c>
+      <c r="N12" t="str">
+        <v>https://nichehire-psi.vercel.app/govt-exams</v>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+      <c r="P12" t="str">
+        <v>New</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>Reported by tester. Active openings count included closed exams, causing dissonance between advertised openings and actual active application windows.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>BUG-009</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Job Search</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Applicant Metric Integrity vs Zero Fake Claim (SRCH-031)</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Search UI retains synthetic "Applicants" filter (&lt;10, &lt;25) and "Early applicant" badges despite "Zero Fake Data" guarantee</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Production (nichehire-psi.vercel.app)</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Candidate searching jobs on homepage / search page</v>
+      </c>
+      <c r="H13" t="str">
+        <v>1. Inspect search filter dropdown "Applicants". 2. Select "Early Bird (&lt; 10)" or "Under 25". 3. Open job details modal for listings without applicant telemetry.</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Platform claiming "Zero Fake Data Guarantee: Real applicants only" should not expose simulated applicant filter brackets or generate synthetic "Early applicant" badges for unverified aggregator/portal jobs.</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Search filter bar retains "Applicants" filter with arbitrary categories (&lt;10, &lt;25, &lt;50) and job details drawer renders synthetic fallback badge "Early applicant" when applicant count is missing.</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="M13" t="str">
+        <v>app/page.tsx:886-892, 2177, CHANGELOG_3_DAYS.md:23</v>
+      </c>
+      <c r="N13" t="str">
+        <v>https://nichehire-psi.vercel.app</v>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+      <c r="P13" t="str">
+        <v>New</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>Reported by tester. Direct conflict between marketing claim of "Zero Fake Data" and UI presence of simulated applicant filter buckets and placeholder badges.</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>BUG-010</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-09-28</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Government Jobs</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Airports Authority Statutory Name Typo (GOV-033)</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Conducting body and section text displays "Airport Authority of India" missing the plural 's'</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Production (nichehire-psi.vercel.app)</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Candidate browsing PSU openings on /govt-exams</v>
+      </c>
+      <c r="H14" t="str">
+        <v>1. Navigate to /govt-exams. 2. Inspect Tier 4 PSU description and conducting body headers for AAI.</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Statutory body rendered accurately as "Airports Authority of India (AAI)".</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Rendered as "Airport Authority of India (AAI)" omitting the statutory 's' in Airports.</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Low</v>
+      </c>
+      <c r="M14" t="str">
+        <v>app/govt-exams/page.tsx:662</v>
+      </c>
+      <c r="N14" t="str">
+        <v>https://nichehire-psi.vercel.app/govt-exams</v>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+      <c r="P14" t="str">
+        <v>New</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>Reported by tester. Minor grammatical/statutory discrepancy in PSU banner copy.</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:Q1"/>

</xml_diff>